<commit_message>
Update NC draft and expand replay-selection diagnostic to 12 schedules
</commit_message>
<xml_diff>
--- a/figure_data/qualification_value/qualification_value.xlsx
+++ b/figure_data/qualification_value/qualification_value.xlsx
@@ -15,7 +15,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Read_me" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fig07_Daily'!$A$1:$K$81</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Fig07_Daily'!$A$1:$T$81</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K81"/>
+  <dimension ref="A1:T81"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -452,9 +452,18 @@
     <col width="21" customWidth="1" min="6" max="6"/>
     <col width="21" customWidth="1" min="7" max="7"/>
     <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="28" customWidth="1" min="9" max="9"/>
-    <col width="28" customWidth="1" min="10" max="10"/>
-    <col width="23" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="9" max="9"/>
+    <col width="21" customWidth="1" min="10" max="10"/>
+    <col width="21" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="21" customWidth="1" min="13" max="13"/>
+    <col width="21" customWidth="1" min="14" max="14"/>
+    <col width="21" customWidth="1" min="15" max="15"/>
+    <col width="21" customWidth="1" min="16" max="16"/>
+    <col width="21" customWidth="1" min="17" max="17"/>
+    <col width="28" customWidth="1" min="18" max="18"/>
+    <col width="28" customWidth="1" min="19" max="19"/>
+    <col width="23" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -495,20 +504,65 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
+          <t>random_2404_mwh</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>random_2405_mwh</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>random_2406_mwh</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>random_2407_mwh</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>random_2408_mwh</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>random_2409_mwh</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>random_2410_mwh</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>random_2411_mwh</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>random_2412_mwh</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
           <t>random_mean_mwh</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>ecf_minus_random_mean_kwh</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>ecf_minus_no_feedback_kwh</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>longest_35_day_block</t>
         </is>
@@ -539,15 +593,42 @@
         <v>3.677545567942218</v>
       </c>
       <c r="H2" s="3" t="n">
-        <v>3.698706528983872</v>
+        <v>3.684921290594112</v>
       </c>
       <c r="I2" s="3" t="n">
-        <v>17.55325245599382</v>
+        <v>3.699071931526984</v>
       </c>
       <c r="J2" s="3" t="n">
+        <v>3.684696553747567</v>
+      </c>
+      <c r="K2" s="3" t="n">
+        <v>3.713649242439645</v>
+      </c>
+      <c r="L2" s="3" t="n">
+        <v>3.691454994457694</v>
+      </c>
+      <c r="M2" s="3" t="n">
+        <v>3.710878615512252</v>
+      </c>
+      <c r="N2" s="3" t="n">
+        <v>3.720597917399717</v>
+      </c>
+      <c r="O2" s="3" t="n">
+        <v>3.677571893352904</v>
+      </c>
+      <c r="P2" s="3" t="n">
+        <v>3.683889190464565</v>
+      </c>
+      <c r="Q2" s="3" t="n">
+        <v>3.696904268037254</v>
+      </c>
+      <c r="R2" s="3" t="n">
+        <v>19.35551340261155</v>
+      </c>
+      <c r="S2" s="3" t="n">
         <v>0.8454056109572505</v>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="T2" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -576,15 +657,42 @@
         <v>4.104478303452973</v>
       </c>
       <c r="H3" s="3" t="n">
-        <v>4.106151443419839</v>
+        <v>4.112055234477834</v>
       </c>
       <c r="I3" s="3" t="n">
-        <v>10.85686588259538</v>
+        <v>4.116411248303278</v>
       </c>
       <c r="J3" s="3" t="n">
+        <v>4.101766120208874</v>
+      </c>
+      <c r="K3" s="3" t="n">
+        <v>4.106083656199115</v>
+      </c>
+      <c r="L3" s="3" t="n">
+        <v>4.112057437932243</v>
+      </c>
+      <c r="M3" s="3" t="n">
+        <v>4.115047009940326</v>
+      </c>
+      <c r="N3" s="3" t="n">
+        <v>4.105416643893556</v>
+      </c>
+      <c r="O3" s="3" t="n">
+        <v>4.106193604184002</v>
+      </c>
+      <c r="P3" s="3" t="n">
+        <v>4.111878439101354</v>
+      </c>
+      <c r="Q3" s="3" t="n">
+        <v>4.108780310375008</v>
+      </c>
+      <c r="R3" s="3" t="n">
+        <v>8.227998927426761</v>
+      </c>
+      <c r="S3" s="3" t="n">
         <v>5.107984360202877</v>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="T3" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -613,15 +721,42 @@
         <v>4.20597714621774</v>
       </c>
       <c r="H4" s="3" t="n">
-        <v>4.203319481050717</v>
+        <v>4.200611294280191</v>
       </c>
       <c r="I4" s="3" t="n">
-        <v>1.97279933654837</v>
+        <v>4.206558635340834</v>
       </c>
       <c r="J4" s="3" t="n">
+        <v>4.195241000897959</v>
+      </c>
+      <c r="K4" s="3" t="n">
+        <v>4.205867914145546</v>
+      </c>
+      <c r="L4" s="3" t="n">
+        <v>4.205176411220292</v>
+      </c>
+      <c r="M4" s="3" t="n">
+        <v>4.206558655409283</v>
+      </c>
+      <c r="N4" s="3" t="n">
+        <v>4.200516780751647</v>
+      </c>
+      <c r="O4" s="3" t="n">
+        <v>4.205161352148447</v>
+      </c>
+      <c r="P4" s="3" t="n">
+        <v>4.20651503057451</v>
+      </c>
+      <c r="Q4" s="3" t="n">
+        <v>4.203513793160071</v>
+      </c>
+      <c r="R4" s="3" t="n">
+        <v>1.778487227194425</v>
+      </c>
+      <c r="S4" s="3" t="n">
         <v>-1.266375022016319</v>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="T4" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -650,15 +785,42 @@
         <v>4.343401710328251</v>
       </c>
       <c r="H5" s="3" t="n">
-        <v>4.341388021451018</v>
+        <v>4.350762470694034</v>
       </c>
       <c r="I5" s="3" t="n">
-        <v>2.937654100009901</v>
+        <v>4.350651351778039</v>
       </c>
       <c r="J5" s="3" t="n">
+        <v>4.326379077335999</v>
+      </c>
+      <c r="K5" s="3" t="n">
+        <v>4.339547093132479</v>
+      </c>
+      <c r="L5" s="3" t="n">
+        <v>4.345960315297791</v>
+      </c>
+      <c r="M5" s="3" t="n">
+        <v>4.344221593178473</v>
+      </c>
+      <c r="N5" s="3" t="n">
+        <v>4.337807934852975</v>
+      </c>
+      <c r="O5" s="3" t="n">
+        <v>4.345762936660609</v>
+      </c>
+      <c r="P5" s="3" t="n">
+        <v>4.347608540221168</v>
+      </c>
+      <c r="Q5" s="3" t="n">
+        <v>4.342738781458719</v>
+      </c>
+      <c r="R5" s="3" t="n">
+        <v>1.586894092309166</v>
+      </c>
+      <c r="S5" s="3" t="n">
         <v>-6.390062940289098</v>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="T5" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -687,15 +849,42 @@
         <v>4.418734436737561</v>
       </c>
       <c r="H6" s="3" t="n">
-        <v>4.456546456405397</v>
+        <v>4.476387784100835</v>
       </c>
       <c r="I6" s="3" t="n">
-        <v>11.84684880177489</v>
+        <v>4.46822136236888</v>
       </c>
       <c r="J6" s="3" t="n">
+        <v>4.464774728377684</v>
+      </c>
+      <c r="K6" s="3" t="n">
+        <v>4.477300157912893</v>
+      </c>
+      <c r="L6" s="3" t="n">
+        <v>4.463201087279081</v>
+      </c>
+      <c r="M6" s="3" t="n">
+        <v>4.474718958961706</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>4.474485466231731</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>4.470652675662795</v>
+      </c>
+      <c r="P6" s="3" t="n">
+        <v>4.470458195090155</v>
+      </c>
+      <c r="Q6" s="3" t="n">
+        <v>4.467486648766829</v>
+      </c>
+      <c r="R6" s="3" t="n">
+        <v>0.9066564403434896</v>
+      </c>
+      <c r="S6" s="3" t="n">
         <v>-8.906866762134591</v>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="T6" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -724,15 +913,42 @@
         <v>4.118999670957398</v>
       </c>
       <c r="H7" s="3" t="n">
-        <v>4.117820343547138</v>
+        <v>4.090229893924604</v>
       </c>
       <c r="I7" s="3" t="n">
-        <v>13.85133561161833</v>
+        <v>4.119373929908295</v>
       </c>
       <c r="J7" s="3" t="n">
+        <v>4.09705738453508</v>
+      </c>
+      <c r="K7" s="3" t="n">
+        <v>4.11936666303889</v>
+      </c>
+      <c r="L7" s="3" t="n">
+        <v>4.106034988164742</v>
+      </c>
+      <c r="M7" s="3" t="n">
+        <v>4.115983557737199</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>4.11928982301325</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>4.11936666303889</v>
+      </c>
+      <c r="P7" s="3" t="n">
+        <v>4.103819536928151</v>
+      </c>
+      <c r="Q7" s="3" t="n">
+        <v>4.111998622577543</v>
+      </c>
+      <c r="R7" s="3" t="n">
+        <v>19.67305658121354</v>
+      </c>
+      <c r="S7" s="3" t="n">
         <v>12.30501611986679</v>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="T7" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -761,15 +977,42 @@
         <v>3.689352585376587</v>
       </c>
       <c r="H8" s="3" t="n">
-        <v>3.69599575660969</v>
+        <v>3.696121067288181</v>
       </c>
       <c r="I8" s="3" t="n">
-        <v>2.513537085608863</v>
+        <v>3.697956617010189</v>
       </c>
       <c r="J8" s="3" t="n">
+        <v>3.700812607554291</v>
+      </c>
+      <c r="K8" s="3" t="n">
+        <v>3.699210225260047</v>
+      </c>
+      <c r="L8" s="3" t="n">
+        <v>3.678999510709466</v>
+      </c>
+      <c r="M8" s="3" t="n">
+        <v>3.690898439875175</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>3.69538978959447</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>3.696724846396124</v>
+      </c>
+      <c r="P8" s="3" t="n">
+        <v>3.69904906737725</v>
+      </c>
+      <c r="Q8" s="3" t="n">
+        <v>3.695262453407855</v>
+      </c>
+      <c r="R8" s="3" t="n">
+        <v>3.246840287443931</v>
+      </c>
+      <c r="S8" s="3" t="n">
         <v>-1.941928183700536</v>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="T8" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -798,15 +1041,42 @@
         <v>3.814724037664181</v>
       </c>
       <c r="H9" s="3" t="n">
-        <v>3.823616492326364</v>
+        <v>3.816369943497698</v>
       </c>
       <c r="I9" s="3" t="n">
-        <v>35.39733070574292</v>
+        <v>3.861060437842711</v>
       </c>
       <c r="J9" s="3" t="n">
+        <v>3.857644222200436</v>
+      </c>
+      <c r="K9" s="3" t="n">
+        <v>3.857916163797008</v>
+      </c>
+      <c r="L9" s="3" t="n">
+        <v>3.83509283644709</v>
+      </c>
+      <c r="M9" s="3" t="n">
+        <v>3.861569842475957</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>3.806595891921248</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>3.849001270603868</v>
+      </c>
+      <c r="P9" s="3" t="n">
+        <v>3.833312042683698</v>
+      </c>
+      <c r="Q9" s="3" t="n">
+        <v>3.837451010704067</v>
+      </c>
+      <c r="R9" s="3" t="n">
+        <v>21.56281232804025</v>
+      </c>
+      <c r="S9" s="3" t="n">
         <v>-2.730610066844275</v>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="T9" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -835,15 +1105,42 @@
         <v>2.815591109109131</v>
       </c>
       <c r="H10" s="3" t="n">
-        <v>2.806981828259515</v>
+        <v>2.795164000612396</v>
       </c>
       <c r="I10" s="3" t="n">
-        <v>23.50375162013707</v>
+        <v>2.806137473353667</v>
       </c>
       <c r="J10" s="3" t="n">
+        <v>2.815865947951512</v>
+      </c>
+      <c r="K10" s="3" t="n">
+        <v>2.803067206997268</v>
+      </c>
+      <c r="L10" s="3" t="n">
+        <v>2.809312564636973</v>
+      </c>
+      <c r="M10" s="3" t="n">
+        <v>2.815370887010301</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>2.816646917424553</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>2.806737585819127</v>
+      </c>
+      <c r="P10" s="3" t="n">
+        <v>2.799736549931846</v>
+      </c>
+      <c r="Q10" s="3" t="n">
+        <v>2.80741538487635</v>
+      </c>
+      <c r="R10" s="3" t="n">
+        <v>23.0701950033021</v>
+      </c>
+      <c r="S10" s="3" t="n">
         <v>23.5881623927221</v>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="T10" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -872,15 +1169,42 @@
         <v>3.869237427211952</v>
       </c>
       <c r="H11" s="3" t="n">
-        <v>3.871862431323373</v>
+        <v>3.866986764038958</v>
       </c>
       <c r="I11" s="3" t="n">
-        <v>1.743729626483059</v>
+        <v>3.868366917481385</v>
       </c>
       <c r="J11" s="3" t="n">
+        <v>3.858454453433601</v>
+      </c>
+      <c r="K11" s="3" t="n">
+        <v>3.869099721852262</v>
+      </c>
+      <c r="L11" s="3" t="n">
+        <v>3.86817837543465</v>
+      </c>
+      <c r="M11" s="3" t="n">
+        <v>3.864965192229569</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>3.869237152402568</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>3.86724078830386</v>
+      </c>
+      <c r="P11" s="3" t="n">
+        <v>3.866650566716872</v>
+      </c>
+      <c r="Q11" s="3" t="n">
+        <v>3.867897268821987</v>
+      </c>
+      <c r="R11" s="3" t="n">
+        <v>5.708892127868737</v>
+      </c>
+      <c r="S11" s="3" t="n">
         <v>4.368733737904584</v>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="T11" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -909,15 +1233,42 @@
         <v>4.13866784384664</v>
       </c>
       <c r="H12" s="3" t="n">
-        <v>4.13872092291788</v>
+        <v>4.122516869718896</v>
       </c>
       <c r="I12" s="3" t="n">
-        <v>43.41848062163223</v>
+        <v>4.144216662738497</v>
       </c>
       <c r="J12" s="3" t="n">
+        <v>4.13867954394088</v>
+      </c>
+      <c r="K12" s="3" t="n">
+        <v>4.138275568166009</v>
+      </c>
+      <c r="L12" s="3" t="n">
+        <v>4.137278444594967</v>
+      </c>
+      <c r="M12" s="3" t="n">
+        <v>4.138654542740253</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>4.144216670903544</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>4.138090287230676</v>
+      </c>
+      <c r="P12" s="3" t="n">
+        <v>4.122345865856783</v>
+      </c>
+      <c r="Q12" s="3" t="n">
+        <v>4.136703102053679</v>
+      </c>
+      <c r="R12" s="3" t="n">
+        <v>45.43630148583322</v>
+      </c>
+      <c r="S12" s="3" t="n">
         <v>43.48486079925973</v>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="T12" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -946,15 +1297,42 @@
         <v>4.104421991980127</v>
       </c>
       <c r="H13" s="3" t="n">
-        <v>4.106860863875144</v>
+        <v>4.113674485913506</v>
       </c>
       <c r="I13" s="3" t="n">
-        <v>5.90803380967575</v>
+        <v>4.112316239723117</v>
       </c>
       <c r="J13" s="3" t="n">
+        <v>4.113429952253821</v>
+      </c>
+      <c r="K13" s="3" t="n">
+        <v>4.109652023153954</v>
+      </c>
+      <c r="L13" s="3" t="n">
+        <v>4.101060722928062</v>
+      </c>
+      <c r="M13" s="3" t="n">
+        <v>4.104252739218185</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>4.113429952253821</v>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>4.110824572484977</v>
+      </c>
+      <c r="P13" s="3" t="n">
+        <v>4.113574951997405</v>
+      </c>
+      <c r="Q13" s="3" t="n">
+        <v>4.109399852629357</v>
+      </c>
+      <c r="R13" s="3" t="n">
+        <v>3.369045055462649</v>
+      </c>
+      <c r="S13" s="3" t="n">
         <v>-0.9055887775852867</v>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="T13" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -983,15 +1361,42 @@
         <v>4.236568329641003</v>
       </c>
       <c r="H14" s="3" t="n">
-        <v>4.236319765828839</v>
+        <v>4.235878748478608</v>
       </c>
       <c r="I14" s="3" t="n">
-        <v>-0.5074463781236105</v>
+        <v>4.236205185687422</v>
       </c>
       <c r="J14" s="3" t="n">
+        <v>4.235527523914951</v>
+      </c>
+      <c r="K14" s="3" t="n">
+        <v>4.224968217165968</v>
+      </c>
+      <c r="L14" s="3" t="n">
+        <v>4.209422546630455</v>
+      </c>
+      <c r="M14" s="3" t="n">
+        <v>4.236205185687422</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>4.235787611037179</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>4.236266478103434</v>
+      </c>
+      <c r="P14" s="3" t="n">
+        <v>4.236176018957807</v>
+      </c>
+      <c r="Q14" s="3" t="n">
+        <v>4.232949734429147</v>
+      </c>
+      <c r="R14" s="3" t="n">
+        <v>2.862585021567554</v>
+      </c>
+      <c r="S14" s="3" t="n">
         <v>-0.3636995070932514</v>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="T14" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1020,15 +1425,42 @@
         <v>3.907844574901112</v>
       </c>
       <c r="H15" s="3" t="n">
-        <v>3.904868923491424</v>
+        <v>3.903398823845886</v>
       </c>
       <c r="I15" s="3" t="n">
-        <v>8.122702449243402</v>
+        <v>3.906603831169507</v>
       </c>
       <c r="J15" s="3" t="n">
+        <v>3.901804228130513</v>
+      </c>
+      <c r="K15" s="3" t="n">
+        <v>3.902002327718524</v>
+      </c>
+      <c r="L15" s="3" t="n">
+        <v>3.903911027838984</v>
+      </c>
+      <c r="M15" s="3" t="n">
+        <v>3.889938867517482</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>3.889993814299697</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>3.908506042855625</v>
+      </c>
+      <c r="P15" s="3" t="n">
+        <v>3.895736213744968</v>
+      </c>
+      <c r="Q15" s="3" t="n">
+        <v>3.901375162299622</v>
+      </c>
+      <c r="R15" s="3" t="n">
+        <v>11.61646364104518</v>
+      </c>
+      <c r="S15" s="3" t="n">
         <v>6.043920571064731</v>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="T15" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1057,15 +1489,42 @@
         <v>3.334324267969701</v>
       </c>
       <c r="H16" s="3" t="n">
-        <v>3.332886703750066</v>
+        <v>3.311532100022499</v>
       </c>
       <c r="I16" s="3" t="n">
-        <v>-10.52947109407576</v>
+        <v>3.334857604157039</v>
       </c>
       <c r="J16" s="3" t="n">
+        <v>3.325763439901315</v>
+      </c>
+      <c r="K16" s="3" t="n">
+        <v>3.324556073431015</v>
+      </c>
+      <c r="L16" s="3" t="n">
+        <v>3.277845772253738</v>
+      </c>
+      <c r="M16" s="3" t="n">
+        <v>3.333693967576909</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>3.325164794459021</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>3.307061828674784</v>
+      </c>
+      <c r="P16" s="3" t="n">
+        <v>3.325448043484417</v>
+      </c>
+      <c r="Q16" s="3" t="n">
+        <v>3.322048644600911</v>
+      </c>
+      <c r="R16" s="3" t="n">
+        <v>0.308588055079273</v>
+      </c>
+      <c r="S16" s="3" t="n">
         <v>-6.922866877327127</v>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="T16" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1094,15 +1553,42 @@
         <v>2.66156521717881</v>
       </c>
       <c r="H17" s="3" t="n">
-        <v>2.657320833009134</v>
+        <v>2.657754415643697</v>
       </c>
       <c r="I17" s="3" t="n">
-        <v>-6.841967912211366</v>
+        <v>2.686240737447236</v>
       </c>
       <c r="J17" s="3" t="n">
+        <v>2.673929815076149</v>
+      </c>
+      <c r="K17" s="3" t="n">
+        <v>2.651155641140829</v>
+      </c>
+      <c r="L17" s="3" t="n">
+        <v>2.681197509035548</v>
+      </c>
+      <c r="M17" s="3" t="n">
+        <v>2.652584244543274</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>2.681650902833508</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>2.66340147905687</v>
+      </c>
+      <c r="P17" s="3" t="n">
+        <v>2.654054658706635</v>
+      </c>
+      <c r="Q17" s="3" t="n">
+        <v>2.664494325209262</v>
+      </c>
+      <c r="R17" s="3" t="n">
+        <v>-14.01546011233945</v>
+      </c>
+      <c r="S17" s="3" t="n">
         <v>-11.08457476096092</v>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="T17" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1131,15 +1617,42 @@
         <v>4.14919739101958</v>
       </c>
       <c r="H18" s="3" t="n">
-        <v>4.14927467785579</v>
+        <v>4.149431399685285</v>
       </c>
       <c r="I18" s="3" t="n">
-        <v>4.097878592907556</v>
+        <v>4.149182663929365</v>
       </c>
       <c r="J18" s="3" t="n">
+        <v>4.149082605455282</v>
+      </c>
+      <c r="K18" s="3" t="n">
+        <v>4.155490822121984</v>
+      </c>
+      <c r="L18" s="3" t="n">
+        <v>4.149182663929365</v>
+      </c>
+      <c r="M18" s="3" t="n">
+        <v>4.149187232067026</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>4.14918250394058</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>4.149280369955703</v>
+      </c>
+      <c r="P18" s="3" t="n">
+        <v>4.158214017186831</v>
+      </c>
+      <c r="Q18" s="3" t="n">
+        <v>4.150504859319899</v>
+      </c>
+      <c r="R18" s="3" t="n">
+        <v>2.867697128798419</v>
+      </c>
+      <c r="S18" s="3" t="n">
         <v>4.189892519333327</v>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="T18" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1168,15 +1681,42 @@
         <v>3.072642207202486</v>
       </c>
       <c r="H19" s="3" t="n">
-        <v>3.059941397583811</v>
+        <v>3.075572967099546</v>
       </c>
       <c r="I19" s="3" t="n">
-        <v>28.90261483593592</v>
+        <v>3.07521661825816</v>
       </c>
       <c r="J19" s="3" t="n">
+        <v>3.085176503100726</v>
+      </c>
+      <c r="K19" s="3" t="n">
+        <v>3.060190247195383</v>
+      </c>
+      <c r="L19" s="3" t="n">
+        <v>3.06755213286577</v>
+      </c>
+      <c r="M19" s="3" t="n">
+        <v>3.07484783927133</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>3.074797036408337</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>3.07356591753407</v>
+      </c>
+      <c r="P19" s="3" t="n">
+        <v>3.072874799117504</v>
+      </c>
+      <c r="Q19" s="3" t="n">
+        <v>3.069968187800189</v>
+      </c>
+      <c r="R19" s="3" t="n">
+        <v>18.87582461955883</v>
+      </c>
+      <c r="S19" s="3" t="n">
         <v>13.27104532020185</v>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="T19" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1205,15 +1745,42 @@
         <v>3.58530911507918</v>
       </c>
       <c r="H20" s="3" t="n">
-        <v>3.584376686774816</v>
+        <v>3.54606978093642</v>
       </c>
       <c r="I20" s="3" t="n">
-        <v>-66.74409146460248</v>
+        <v>3.579992383066636</v>
       </c>
       <c r="J20" s="3" t="n">
+        <v>3.556295118297769</v>
+      </c>
+      <c r="K20" s="3" t="n">
+        <v>3.561527587814519</v>
+      </c>
+      <c r="L20" s="3" t="n">
+        <v>3.554829706615415</v>
+      </c>
+      <c r="M20" s="3" t="n">
+        <v>3.565456309892698</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>3.546379737594625</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>3.580272370083451</v>
+      </c>
+      <c r="P20" s="3" t="n">
+        <v>3.560083603894852</v>
+      </c>
+      <c r="Q20" s="3" t="n">
+        <v>3.567003054876736</v>
+      </c>
+      <c r="R20" s="3" t="n">
+        <v>-49.37045956652275</v>
+      </c>
+      <c r="S20" s="3" t="n">
         <v>-67.93918865368641</v>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="T20" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1242,15 +1809,42 @@
         <v>4.139356170999887</v>
       </c>
       <c r="H21" s="3" t="n">
-        <v>4.151546618333559</v>
+        <v>4.161406017590799</v>
       </c>
       <c r="I21" s="3" t="n">
-        <v>15.74842635794393</v>
+        <v>4.121946782049397</v>
       </c>
       <c r="J21" s="3" t="n">
+        <v>4.139958770948724</v>
+      </c>
+      <c r="K21" s="3" t="n">
+        <v>4.140101544506827</v>
+      </c>
+      <c r="L21" s="3" t="n">
+        <v>4.140003462139193</v>
+      </c>
+      <c r="M21" s="3" t="n">
+        <v>4.140729921039653</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>4.141496026012921</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>4.143728265758902</v>
+      </c>
+      <c r="P21" s="3" t="n">
+        <v>4.136568419673758</v>
+      </c>
+      <c r="Q21" s="3" t="n">
+        <v>4.143381588726737</v>
+      </c>
+      <c r="R21" s="3" t="n">
+        <v>23.9134559647658</v>
+      </c>
+      <c r="S21" s="3" t="n">
         <v>27.21986926702868</v>
       </c>
-      <c r="K21" s="2" t="n">
+      <c r="T21" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1279,15 +1873,42 @@
         <v>3.9852038175589</v>
       </c>
       <c r="H22" s="3" t="n">
-        <v>3.981119195350038</v>
+        <v>3.985203840608341</v>
       </c>
       <c r="I22" s="3" t="n">
-        <v>-10.40046557856034</v>
+        <v>3.985203840437998</v>
       </c>
       <c r="J22" s="3" t="n">
+        <v>3.972485227484806</v>
+      </c>
+      <c r="K22" s="3" t="n">
+        <v>3.984912074205198</v>
+      </c>
+      <c r="L22" s="3" t="n">
+        <v>3.974209053894226</v>
+      </c>
+      <c r="M22" s="3" t="n">
+        <v>3.978812378050887</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>4.030606271488824</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>3.979864965423587</v>
+      </c>
+      <c r="P22" s="3" t="n">
+        <v>3.986981557477463</v>
+      </c>
+      <c r="Q22" s="3" t="n">
+        <v>3.985136399593454</v>
+      </c>
+      <c r="R22" s="3" t="n">
+        <v>-14.41766982197645</v>
+      </c>
+      <c r="S22" s="3" t="n">
         <v>-14.4851108718238</v>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="T22" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1316,15 +1937,42 @@
         <v>3.354239835222897</v>
       </c>
       <c r="H23" s="3" t="n">
-        <v>3.354790480070314</v>
+        <v>3.352735949100164</v>
       </c>
       <c r="I23" s="3" t="n">
-        <v>1.037035578260959</v>
+        <v>3.355135417165709</v>
       </c>
       <c r="J23" s="3" t="n">
+        <v>3.352385483750958</v>
+      </c>
+      <c r="K23" s="3" t="n">
+        <v>3.350664919707796</v>
+      </c>
+      <c r="L23" s="3" t="n">
+        <v>3.362567185005493</v>
+      </c>
+      <c r="M23" s="3" t="n">
+        <v>3.35448172091729</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>3.354585285187995</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>3.349137899889866</v>
+      </c>
+      <c r="P23" s="3" t="n">
+        <v>3.354853786475708</v>
+      </c>
+      <c r="Q23" s="3" t="n">
+        <v>3.354243257284327</v>
+      </c>
+      <c r="R23" s="3" t="n">
+        <v>1.584258364248026</v>
+      </c>
+      <c r="S23" s="3" t="n">
         <v>0.6920984828657772</v>
       </c>
-      <c r="K23" s="2" t="n">
+      <c r="T23" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1353,15 +2001,42 @@
         <v>1.986695470020964</v>
       </c>
       <c r="H24" s="3" t="n">
-        <v>2.004246211956885</v>
+        <v>2.060725654602625</v>
       </c>
       <c r="I24" s="3" t="n">
-        <v>141.2766221642232</v>
+        <v>2.04327401053138</v>
       </c>
       <c r="J24" s="3" t="n">
+        <v>2.021113943950263</v>
+      </c>
+      <c r="K24" s="3" t="n">
+        <v>2.037207465555704</v>
+      </c>
+      <c r="L24" s="3" t="n">
+        <v>2.0017313548684</v>
+      </c>
+      <c r="M24" s="3" t="n">
+        <v>2.084630019042685</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>2.066267360982793</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>2.071568548378052</v>
+      </c>
+      <c r="P24" s="3" t="n">
+        <v>2.096306329959056</v>
+      </c>
+      <c r="Q24" s="3" t="n">
+        <v>2.041296943645134</v>
+      </c>
+      <c r="R24" s="3" t="n">
+        <v>104.2258904759739</v>
+      </c>
+      <c r="S24" s="3" t="n">
         <v>60.89282936468798</v>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="T24" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1390,15 +2065,42 @@
         <v>2.947319044726276</v>
       </c>
       <c r="H25" s="3" t="n">
-        <v>2.947365513295953</v>
+        <v>2.945774395130213</v>
       </c>
       <c r="I25" s="3" t="n">
-        <v>-0.3410635516969407</v>
+        <v>2.94768842468245</v>
       </c>
       <c r="J25" s="3" t="n">
+        <v>2.947487422423417</v>
+      </c>
+      <c r="K25" s="3" t="n">
+        <v>2.947361620311616</v>
+      </c>
+      <c r="L25" s="3" t="n">
+        <v>2.946223922470163</v>
+      </c>
+      <c r="M25" s="3" t="n">
+        <v>2.947094254994052</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>2.9285226894443</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>2.947204409015732</v>
+      </c>
+      <c r="P25" s="3" t="n">
+        <v>2.939469821074499</v>
+      </c>
+      <c r="Q25" s="3" t="n">
+        <v>2.944910291619525</v>
+      </c>
+      <c r="R25" s="3" t="n">
+        <v>2.114158124730814</v>
+      </c>
+      <c r="S25" s="3" t="n">
         <v>-0.3871333192657644</v>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="T25" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1427,15 +2129,42 @@
         <v>2.891390561414779</v>
       </c>
       <c r="H26" s="3" t="n">
-        <v>2.938173983138892</v>
+        <v>3.010529755930104</v>
       </c>
       <c r="I26" s="3" t="n">
-        <v>92.30503088966825</v>
+        <v>2.979561625834059</v>
       </c>
       <c r="J26" s="3" t="n">
+        <v>2.896704477771639</v>
+      </c>
+      <c r="K26" s="3" t="n">
+        <v>3.009066894150397</v>
+      </c>
+      <c r="L26" s="3" t="n">
+        <v>2.913505555071694</v>
+      </c>
+      <c r="M26" s="3" t="n">
+        <v>2.918987044540502</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>2.867303278974112</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>2.982597801797559</v>
+      </c>
+      <c r="P26" s="3" t="n">
+        <v>2.902658106714258</v>
+      </c>
+      <c r="Q26" s="3" t="n">
+        <v>2.941286374183417</v>
+      </c>
+      <c r="R26" s="3" t="n">
+        <v>89.19263984514414</v>
+      </c>
+      <c r="S26" s="3" t="n">
         <v>115.387520950831</v>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="T26" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1464,15 +2193,42 @@
         <v>3.823267221764531</v>
       </c>
       <c r="H27" s="3" t="n">
-        <v>3.821951152782677</v>
+        <v>3.824144722157244</v>
       </c>
       <c r="I27" s="3" t="n">
-        <v>-0.2546245074923625</v>
+        <v>3.822763445166747</v>
       </c>
       <c r="J27" s="3" t="n">
+        <v>3.823618832107986</v>
+      </c>
+      <c r="K27" s="3" t="n">
+        <v>3.821546539302549</v>
+      </c>
+      <c r="L27" s="3" t="n">
+        <v>3.822589834970743</v>
+      </c>
+      <c r="M27" s="3" t="n">
+        <v>3.824943710796278</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>3.811894134827541</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>3.82432528763023</v>
+      </c>
+      <c r="P27" s="3" t="n">
+        <v>3.824919171539805</v>
+      </c>
+      <c r="Q27" s="3" t="n">
+        <v>3.822216594737263</v>
+      </c>
+      <c r="R27" s="3" t="n">
+        <v>-0.5200664620779172</v>
+      </c>
+      <c r="S27" s="3" t="n">
         <v>-3.655305298572387</v>
       </c>
-      <c r="K27" s="2" t="n">
+      <c r="T27" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1501,15 +2257,42 @@
         <v>3.405311962563819</v>
       </c>
       <c r="H28" s="3" t="n">
-        <v>3.404116584787717</v>
+        <v>3.405120380911765</v>
       </c>
       <c r="I28" s="3" t="n">
-        <v>3.070958400753998</v>
+        <v>3.404775665961039</v>
       </c>
       <c r="J28" s="3" t="n">
+        <v>3.406848449331671</v>
+      </c>
+      <c r="K28" s="3" t="n">
+        <v>3.407264827519726</v>
+      </c>
+      <c r="L28" s="3" t="n">
+        <v>3.398628133104728</v>
+      </c>
+      <c r="M28" s="3" t="n">
+        <v>3.404800891669616</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>3.405038802830118</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>3.40651051468563</v>
+      </c>
+      <c r="P28" s="3" t="n">
+        <v>3.40752690734849</v>
+      </c>
+      <c r="Q28" s="3" t="n">
+        <v>3.404905360643828</v>
+      </c>
+      <c r="R28" s="3" t="n">
+        <v>2.282182544643074</v>
+      </c>
+      <c r="S28" s="3" t="n">
         <v>-0.07728433125508971</v>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="T28" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1538,15 +2321,42 @@
         <v>3.301827574213114</v>
       </c>
       <c r="H29" s="3" t="n">
-        <v>3.290782993791229</v>
+        <v>3.252530470449285</v>
       </c>
       <c r="I29" s="3" t="n">
-        <v>15.06649031011786</v>
+        <v>3.299823499662234</v>
       </c>
       <c r="J29" s="3" t="n">
+        <v>3.301589693964062</v>
+      </c>
+      <c r="K29" s="3" t="n">
+        <v>3.296071530398969</v>
+      </c>
+      <c r="L29" s="3" t="n">
+        <v>3.301881791076575</v>
+      </c>
+      <c r="M29" s="3" t="n">
+        <v>3.296126035503895</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>3.249831960325207</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>3.300824157429592</v>
+      </c>
+      <c r="P29" s="3" t="n">
+        <v>3.278972654592279</v>
+      </c>
+      <c r="Q29" s="3" t="n">
+        <v>3.28750006456465</v>
+      </c>
+      <c r="R29" s="3" t="n">
+        <v>18.34941953669755</v>
+      </c>
+      <c r="S29" s="3" t="n">
         <v>3.974023924480097</v>
       </c>
-      <c r="K29" s="2" t="n">
+      <c r="T29" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1575,15 +2385,42 @@
         <v>2.900374266874421</v>
       </c>
       <c r="H30" s="3" t="n">
-        <v>2.912031629237311</v>
+        <v>2.918364298717291</v>
       </c>
       <c r="I30" s="3" t="n">
-        <v>-115.8364226780866</v>
+        <v>2.918432043827733</v>
       </c>
       <c r="J30" s="3" t="n">
+        <v>2.918641868879671</v>
+      </c>
+      <c r="K30" s="3" t="n">
+        <v>2.917975588636982</v>
+      </c>
+      <c r="L30" s="3" t="n">
+        <v>2.91823520107602</v>
+      </c>
+      <c r="M30" s="3" t="n">
+        <v>2.909221895825652</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>2.918795305848657</v>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>2.82590566070323</v>
+      </c>
+      <c r="P30" s="3" t="n">
+        <v>2.918521145501987</v>
+      </c>
+      <c r="Q30" s="3" t="n">
+        <v>2.908348991394097</v>
+      </c>
+      <c r="R30" s="3" t="n">
+        <v>-112.1537848348733</v>
+      </c>
+      <c r="S30" s="3" t="n">
         <v>-122.4469208566408</v>
       </c>
-      <c r="K30" s="2" t="n">
+      <c r="T30" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1612,15 +2449,42 @@
         <v>3.165891185753929</v>
       </c>
       <c r="H31" s="3" t="n">
-        <v>3.171579808389301</v>
+        <v>3.171809143615981</v>
       </c>
       <c r="I31" s="3" t="n">
-        <v>5.829216172842155</v>
+        <v>3.173801829539384</v>
       </c>
       <c r="J31" s="3" t="n">
+        <v>3.172882832818479</v>
+      </c>
+      <c r="K31" s="3" t="n">
+        <v>3.169759147437925</v>
+      </c>
+      <c r="L31" s="3" t="n">
+        <v>3.175056433741186</v>
+      </c>
+      <c r="M31" s="3" t="n">
+        <v>3.161199956562958</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>3.174078766262808</v>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>3.166264676599652</v>
+      </c>
+      <c r="P31" s="3" t="n">
+        <v>3.171929130403169</v>
+      </c>
+      <c r="Q31" s="3" t="n">
+        <v>3.170960111845787</v>
+      </c>
+      <c r="R31" s="3" t="n">
+        <v>6.448912716356059</v>
+      </c>
+      <c r="S31" s="3" t="n">
         <v>2.352590820957179</v>
       </c>
-      <c r="K31" s="2" t="n">
+      <c r="T31" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1649,15 +2513,42 @@
         <v>3.221620253003841</v>
       </c>
       <c r="H32" s="3" t="n">
-        <v>3.221913560072627</v>
+        <v>3.221950053576849</v>
       </c>
       <c r="I32" s="3" t="n">
-        <v>-3.953301207437754</v>
+        <v>3.219118010362284</v>
       </c>
       <c r="J32" s="3" t="n">
+        <v>3.219276387508399</v>
+      </c>
+      <c r="K32" s="3" t="n">
+        <v>3.222060090406053</v>
+      </c>
+      <c r="L32" s="3" t="n">
+        <v>3.215748257686526</v>
+      </c>
+      <c r="M32" s="3" t="n">
+        <v>3.222060115740791</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>3.220258108835538</v>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>3.213440889273323</v>
+      </c>
+      <c r="P32" s="3" t="n">
+        <v>3.220136562947695</v>
+      </c>
+      <c r="Q32" s="3" t="n">
+        <v>3.219982429712945</v>
+      </c>
+      <c r="R32" s="3" t="n">
+        <v>-2.022170847755689</v>
+      </c>
+      <c r="S32" s="3" t="n">
         <v>-4.099979827049793</v>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="T32" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1686,15 +2577,42 @@
         <v>2.818880216797633</v>
       </c>
       <c r="H33" s="3" t="n">
-        <v>2.807482245958598</v>
+        <v>2.810072814966862</v>
       </c>
       <c r="I33" s="3" t="n">
-        <v>-13.60835680102257</v>
+        <v>2.805251865832849</v>
       </c>
       <c r="J33" s="3" t="n">
+        <v>2.805163777684878</v>
+      </c>
+      <c r="K33" s="3" t="n">
+        <v>2.812226687639181</v>
+      </c>
+      <c r="L33" s="3" t="n">
+        <v>2.784102890049483</v>
+      </c>
+      <c r="M33" s="3" t="n">
+        <v>2.807530670464364</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>2.812784181865716</v>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>2.808325057895448</v>
+      </c>
+      <c r="P33" s="3" t="n">
+        <v>2.807366011883049</v>
+      </c>
+      <c r="Q33" s="3" t="n">
+        <v>2.806272558013136</v>
+      </c>
+      <c r="R33" s="3" t="n">
+        <v>-12.39866885555996</v>
+      </c>
+      <c r="S33" s="3" t="n">
         <v>-14.74953369128418</v>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="T33" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1723,15 +2641,42 @@
         <v>3.147346138165052</v>
       </c>
       <c r="H34" s="3" t="n">
-        <v>3.146279513015298</v>
+        <v>3.144078145312796</v>
       </c>
       <c r="I34" s="3" t="n">
-        <v>-0.4717127736912907</v>
+        <v>3.146636754637871</v>
       </c>
       <c r="J34" s="3" t="n">
+        <v>3.137391515401244</v>
+      </c>
+      <c r="K34" s="3" t="n">
+        <v>3.147737236562804</v>
+      </c>
+      <c r="L34" s="3" t="n">
+        <v>3.146617524137274</v>
+      </c>
+      <c r="M34" s="3" t="n">
+        <v>3.146636754637871</v>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>3.146636754637871</v>
+      </c>
+      <c r="O34" s="3" t="n">
+        <v>3.144660550640411</v>
+      </c>
+      <c r="P34" s="3" t="n">
+        <v>3.144121632324974</v>
+      </c>
+      <c r="Q34" s="3" t="n">
+        <v>3.145279617278251</v>
+      </c>
+      <c r="R34" s="3" t="n">
+        <v>0.5281829633556612</v>
+      </c>
+      <c r="S34" s="3" t="n">
         <v>-0.8289543962645141</v>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="T34" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1760,15 +2705,42 @@
         <v>3.007562767447799</v>
       </c>
       <c r="H35" s="3" t="n">
-        <v>3.005121908593313</v>
+        <v>3.007304320499699</v>
       </c>
       <c r="I35" s="3" t="n">
-        <v>2.139989977600898</v>
+        <v>3.006303466629567</v>
       </c>
       <c r="J35" s="3" t="n">
+        <v>3.007493323640413</v>
+      </c>
+      <c r="K35" s="3" t="n">
+        <v>3.000566788169746</v>
+      </c>
+      <c r="L35" s="3" t="n">
+        <v>3.006867445342903</v>
+      </c>
+      <c r="M35" s="3" t="n">
+        <v>3.007329825948851</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>3.007329060130288</v>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>3.006368875713266</v>
+      </c>
+      <c r="P35" s="3" t="n">
+        <v>3.006955764208749</v>
+      </c>
+      <c r="Q35" s="3" t="n">
+        <v>3.005990383005285</v>
+      </c>
+      <c r="R35" s="3" t="n">
+        <v>1.271515565629322</v>
+      </c>
+      <c r="S35" s="3" t="n">
         <v>-0.3008688768848522</v>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="T35" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1797,15 +2769,42 @@
         <v>2.90754051420308</v>
       </c>
       <c r="H36" s="3" t="n">
-        <v>2.908474512141545</v>
+        <v>2.907244727433216</v>
       </c>
       <c r="I36" s="3" t="n">
-        <v>29.39988359406209</v>
+        <v>2.907429216689037</v>
       </c>
       <c r="J36" s="3" t="n">
+        <v>2.909101843644633</v>
+      </c>
+      <c r="K36" s="3" t="n">
+        <v>2.907853806318377</v>
+      </c>
+      <c r="L36" s="3" t="n">
+        <v>2.910581459860535</v>
+      </c>
+      <c r="M36" s="3" t="n">
+        <v>2.904898383162996</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>2.907854579456666</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>2.900594861236192</v>
+      </c>
+      <c r="P36" s="3" t="n">
+        <v>2.90433114037888</v>
+      </c>
+      <c r="Q36" s="3" t="n">
+        <v>2.907109462883764</v>
+      </c>
+      <c r="R36" s="3" t="n">
+        <v>30.7649328518429</v>
+      </c>
+      <c r="S36" s="3" t="n">
         <v>27.31427584077606</v>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="T36" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1834,15 +2833,42 @@
         <v>3.069402678840484</v>
       </c>
       <c r="H37" s="3" t="n">
-        <v>3.069766261189738</v>
+        <v>3.070088944521491</v>
       </c>
       <c r="I37" s="3" t="n">
-        <v>0.424570524736545</v>
+        <v>3.055609200502013</v>
       </c>
       <c r="J37" s="3" t="n">
+        <v>3.069135023012645</v>
+      </c>
+      <c r="K37" s="3" t="n">
+        <v>3.070082035425385</v>
+      </c>
+      <c r="L37" s="3" t="n">
+        <v>3.08557257720729</v>
+      </c>
+      <c r="M37" s="3" t="n">
+        <v>3.071890782291697</v>
+      </c>
+      <c r="N37" s="3" t="n">
+        <v>3.064371630985027</v>
+      </c>
+      <c r="O37" s="3" t="n">
+        <v>3.069364186832837</v>
+      </c>
+      <c r="P37" s="3" t="n">
+        <v>3.07037659564826</v>
+      </c>
+      <c r="Q37" s="3" t="n">
+        <v>3.069649146666322</v>
+      </c>
+      <c r="R37" s="3" t="n">
+        <v>0.5416850481525515</v>
+      </c>
+      <c r="S37" s="3" t="n">
         <v>-0.1857639337856654</v>
       </c>
-      <c r="K37" s="2" t="n">
+      <c r="T37" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1871,15 +2897,42 @@
         <v>3.107526282682533</v>
       </c>
       <c r="H38" s="3" t="n">
-        <v>3.105550057831294</v>
+        <v>3.104108220986312</v>
       </c>
       <c r="I38" s="3" t="n">
-        <v>2.929198674646916</v>
+        <v>3.09819839237534</v>
       </c>
       <c r="J38" s="3" t="n">
+        <v>3.107130166299832</v>
+      </c>
+      <c r="K38" s="3" t="n">
+        <v>3.107917195575848</v>
+      </c>
+      <c r="L38" s="3" t="n">
+        <v>3.106669724904827</v>
+      </c>
+      <c r="M38" s="3" t="n">
+        <v>3.106351307024725</v>
+      </c>
+      <c r="N38" s="3" t="n">
+        <v>3.105605597303901</v>
+      </c>
+      <c r="O38" s="3" t="n">
+        <v>3.094067935589885</v>
+      </c>
+      <c r="P38" s="3" t="n">
+        <v>3.107827110043972</v>
+      </c>
+      <c r="Q38" s="3" t="n">
+        <v>3.10454381863321</v>
+      </c>
+      <c r="R38" s="3" t="n">
+        <v>3.935437872731207</v>
+      </c>
+      <c r="S38" s="3" t="n">
         <v>-0.2866176477667182</v>
       </c>
-      <c r="K38" s="2" t="n">
+      <c r="T38" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1908,15 +2961,42 @@
         <v>3.002478174568617</v>
       </c>
       <c r="H39" s="3" t="n">
-        <v>3.006903498237024</v>
+        <v>3.003638950504722</v>
       </c>
       <c r="I39" s="3" t="n">
-        <v>0.4873232991609022</v>
+        <v>3.003097745394578</v>
       </c>
       <c r="J39" s="3" t="n">
+        <v>3.013301935862045</v>
+      </c>
+      <c r="K39" s="3" t="n">
+        <v>3.003549430121791</v>
+      </c>
+      <c r="L39" s="3" t="n">
+        <v>3.003285259113674</v>
+      </c>
+      <c r="M39" s="3" t="n">
+        <v>3.006791607547385</v>
+      </c>
+      <c r="N39" s="3" t="n">
+        <v>3.005493804440404</v>
+      </c>
+      <c r="O39" s="3" t="n">
+        <v>3.003979236541399</v>
+      </c>
+      <c r="P39" s="3" t="n">
+        <v>3.005898777858309</v>
+      </c>
+      <c r="Q39" s="3" t="n">
+        <v>3.005812270174614</v>
+      </c>
+      <c r="R39" s="3" t="n">
+        <v>1.578551361570479</v>
+      </c>
+      <c r="S39" s="3" t="n">
         <v>1.492007536052498</v>
       </c>
-      <c r="K39" s="2" t="n">
+      <c r="T39" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1945,15 +3025,42 @@
         <v>2.63552997783348</v>
       </c>
       <c r="H40" s="3" t="n">
-        <v>2.640498448117887</v>
+        <v>2.64409349554491</v>
       </c>
       <c r="I40" s="3" t="n">
-        <v>193.3566953389518</v>
+        <v>2.677669425640279</v>
       </c>
       <c r="J40" s="3" t="n">
+        <v>2.701131023433015</v>
+      </c>
+      <c r="K40" s="3" t="n">
+        <v>2.68520460125136</v>
+      </c>
+      <c r="L40" s="3" t="n">
+        <v>2.700025251132627</v>
+      </c>
+      <c r="M40" s="3" t="n">
+        <v>2.782593986098469</v>
+      </c>
+      <c r="N40" s="3" t="n">
+        <v>2.714180953878594</v>
+      </c>
+      <c r="O40" s="3" t="n">
+        <v>2.71916071609956</v>
+      </c>
+      <c r="P40" s="3" t="n">
+        <v>2.67993016198728</v>
+      </c>
+      <c r="Q40" s="3" t="n">
+        <v>2.685457079951646</v>
+      </c>
+      <c r="R40" s="3" t="n">
+        <v>148.3980635051929</v>
+      </c>
+      <c r="S40" s="3" t="n">
         <v>181.3713723184032</v>
       </c>
-      <c r="K40" s="2" t="n">
+      <c r="T40" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1982,15 +3089,42 @@
         <v>3.424892328931651</v>
       </c>
       <c r="H41" s="3" t="n">
-        <v>3.421924141336863</v>
+        <v>3.418382776417555</v>
       </c>
       <c r="I41" s="3" t="n">
-        <v>1.44113581766403</v>
+        <v>3.424493272727066</v>
       </c>
       <c r="J41" s="3" t="n">
+        <v>3.423805532274824</v>
+      </c>
+      <c r="K41" s="3" t="n">
+        <v>3.424895487741849</v>
+      </c>
+      <c r="L41" s="3" t="n">
+        <v>3.427083780615688</v>
+      </c>
+      <c r="M41" s="3" t="n">
+        <v>3.423619963929139</v>
+      </c>
+      <c r="N41" s="3" t="n">
+        <v>3.423971570801367</v>
+      </c>
+      <c r="O41" s="3" t="n">
+        <v>3.426226499110996</v>
+      </c>
+      <c r="P41" s="3" t="n">
+        <v>3.424882425386527</v>
+      </c>
+      <c r="Q41" s="3" t="n">
+        <v>3.4235944777513</v>
+      </c>
+      <c r="R41" s="3" t="n">
+        <v>-0.2292005967725608</v>
+      </c>
+      <c r="S41" s="3" t="n">
         <v>-1.527052810296858</v>
       </c>
-      <c r="K41" s="2" t="n">
+      <c r="T41" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -2019,15 +3153,42 @@
         <v>2.867810164207238</v>
       </c>
       <c r="H42" s="3" t="n">
-        <v>2.943913648930783</v>
+        <v>2.87471195629759</v>
       </c>
       <c r="I42" s="3" t="n">
-        <v>51.96923554615074</v>
+        <v>2.879700790607343</v>
       </c>
       <c r="J42" s="3" t="n">
+        <v>2.877397924117465</v>
+      </c>
+      <c r="K42" s="3" t="n">
+        <v>2.875561983500567</v>
+      </c>
+      <c r="L42" s="3" t="n">
+        <v>2.876363520851091</v>
+      </c>
+      <c r="M42" s="3" t="n">
+        <v>2.866747082653599</v>
+      </c>
+      <c r="N42" s="3" t="n">
+        <v>2.993981027642235</v>
+      </c>
+      <c r="O42" s="3" t="n">
+        <v>2.868639004115945</v>
+      </c>
+      <c r="P42" s="3" t="n">
+        <v>2.859367912019717</v>
+      </c>
+      <c r="Q42" s="3" t="n">
+        <v>2.900351012383158</v>
+      </c>
+      <c r="R42" s="3" t="n">
+        <v>95.53187209377523</v>
+      </c>
+      <c r="S42" s="3" t="n">
         <v>110.8535075440353</v>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="T42" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2056,15 +3217,42 @@
         <v>2.939604797217463</v>
       </c>
       <c r="H43" s="3" t="n">
-        <v>2.938265248672536</v>
+        <v>2.939739548456233</v>
       </c>
       <c r="I43" s="3" t="n">
-        <v>2.329235408725427</v>
+        <v>2.937737301590509</v>
       </c>
       <c r="J43" s="3" t="n">
+        <v>2.94133605341526</v>
+      </c>
+      <c r="K43" s="3" t="n">
+        <v>2.930097502653961</v>
+      </c>
+      <c r="L43" s="3" t="n">
+        <v>2.939655682077781</v>
+      </c>
+      <c r="M43" s="3" t="n">
+        <v>2.940388314051618</v>
+      </c>
+      <c r="N43" s="3" t="n">
+        <v>2.941155539143915</v>
+      </c>
+      <c r="O43" s="3" t="n">
+        <v>2.940072324821361</v>
+      </c>
+      <c r="P43" s="3" t="n">
+        <v>2.937555588621952</v>
+      </c>
+      <c r="Q43" s="3" t="n">
+        <v>2.938544466737516</v>
+      </c>
+      <c r="R43" s="3" t="n">
+        <v>2.05001734374477</v>
+      </c>
+      <c r="S43" s="3" t="n">
         <v>0.6143753504721516</v>
       </c>
-      <c r="K43" s="2" t="n">
+      <c r="T43" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2093,15 +3281,42 @@
         <v>2.932995122626755</v>
       </c>
       <c r="H44" s="3" t="n">
-        <v>2.916744657237781</v>
+        <v>2.923283035080309</v>
       </c>
       <c r="I44" s="3" t="n">
-        <v>10.38949809707423</v>
+        <v>2.931332662444749</v>
       </c>
       <c r="J44" s="3" t="n">
+        <v>2.933532952840967</v>
+      </c>
+      <c r="K44" s="3" t="n">
+        <v>2.905747631217181</v>
+      </c>
+      <c r="L44" s="3" t="n">
+        <v>2.917505892650692</v>
+      </c>
+      <c r="M44" s="3" t="n">
+        <v>2.923983398669969</v>
+      </c>
+      <c r="N44" s="3" t="n">
+        <v>2.921557054619848</v>
+      </c>
+      <c r="O44" s="3" t="n">
+        <v>2.91747919806353</v>
+      </c>
+      <c r="P44" s="3" t="n">
+        <v>2.925859977531485</v>
+      </c>
+      <c r="Q44" s="3" t="n">
+        <v>2.92087631456934</v>
+      </c>
+      <c r="R44" s="3" t="n">
+        <v>6.257840765515166</v>
+      </c>
+      <c r="S44" s="3" t="n">
         <v>0.345250565450872</v>
       </c>
-      <c r="K44" s="2" t="n">
+      <c r="T44" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2130,15 +3345,42 @@
         <v>2.884519540785488</v>
       </c>
       <c r="H45" s="3" t="n">
-        <v>2.883151713676157</v>
+        <v>2.889894127000511</v>
       </c>
       <c r="I45" s="3" t="n">
-        <v>8.546777828508656</v>
+        <v>2.900839784260298</v>
       </c>
       <c r="J45" s="3" t="n">
+        <v>2.88889126926107</v>
+      </c>
+      <c r="K45" s="3" t="n">
+        <v>2.882104684536865</v>
+      </c>
+      <c r="L45" s="3" t="n">
+        <v>2.890914573044833</v>
+      </c>
+      <c r="M45" s="3" t="n">
+        <v>2.897429782124429</v>
+      </c>
+      <c r="N45" s="3" t="n">
+        <v>2.890927802892352</v>
+      </c>
+      <c r="O45" s="3" t="n">
+        <v>2.890441834262715</v>
+      </c>
+      <c r="P45" s="3" t="n">
+        <v>2.890543143251711</v>
+      </c>
+      <c r="Q45" s="3" t="n">
+        <v>2.889286845138605</v>
+      </c>
+      <c r="R45" s="3" t="n">
+        <v>2.411646366060616</v>
+      </c>
+      <c r="S45" s="3" t="n">
         <v>0.7838999987797024</v>
       </c>
-      <c r="K45" s="2" t="n">
+      <c r="T45" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2167,15 +3409,42 @@
         <v>2.806956111904154</v>
       </c>
       <c r="H46" s="3" t="n">
-        <v>2.807390135142291</v>
+        <v>2.81224945939067</v>
       </c>
       <c r="I46" s="3" t="n">
-        <v>3.219128483553657</v>
+        <v>2.799697218200643</v>
       </c>
       <c r="J46" s="3" t="n">
+        <v>2.803918286367183</v>
+      </c>
+      <c r="K46" s="3" t="n">
+        <v>2.804337459651072</v>
+      </c>
+      <c r="L46" s="3" t="n">
+        <v>2.801857688017088</v>
+      </c>
+      <c r="M46" s="3" t="n">
+        <v>2.80609417477609</v>
+      </c>
+      <c r="N46" s="3" t="n">
+        <v>2.806663645519919</v>
+      </c>
+      <c r="O46" s="3" t="n">
+        <v>2.813634473360378</v>
+      </c>
+      <c r="P46" s="3" t="n">
+        <v>2.809076089566762</v>
+      </c>
+      <c r="Q46" s="3" t="n">
+        <v>2.806641575023056</v>
+      </c>
+      <c r="R46" s="3" t="n">
+        <v>3.967688602788844</v>
+      </c>
+      <c r="S46" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K46" s="2" t="n">
+      <c r="T46" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2204,15 +3473,42 @@
         <v>2.819570078220461</v>
       </c>
       <c r="H47" s="3" t="n">
-        <v>2.819530216507589</v>
+        <v>2.81236997112419</v>
       </c>
       <c r="I47" s="3" t="n">
-        <v>4.276107608142787</v>
+        <v>2.821232797879607</v>
       </c>
       <c r="J47" s="3" t="n">
+        <v>2.822588921018062</v>
+      </c>
+      <c r="K47" s="3" t="n">
+        <v>2.807088050402694</v>
+      </c>
+      <c r="L47" s="3" t="n">
+        <v>2.823158205759013</v>
+      </c>
+      <c r="M47" s="3" t="n">
+        <v>2.823788292173093</v>
+      </c>
+      <c r="N47" s="3" t="n">
+        <v>2.822201539821615</v>
+      </c>
+      <c r="O47" s="3" t="n">
+        <v>2.8170735255924</v>
+      </c>
+      <c r="P47" s="3" t="n">
+        <v>2.821448619167644</v>
+      </c>
+      <c r="Q47" s="3" t="n">
+        <v>2.819128381038424</v>
+      </c>
+      <c r="R47" s="3" t="n">
+        <v>4.677943077308289</v>
+      </c>
+      <c r="S47" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K47" s="2" t="n">
+      <c r="T47" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2241,15 +3537,42 @@
         <v>1.997570302039458</v>
       </c>
       <c r="H48" s="3" t="n">
-        <v>1.986706567068247</v>
+        <v>2.006073811457594</v>
       </c>
       <c r="I48" s="3" t="n">
-        <v>20.19915931879645</v>
+        <v>1.984016951476768</v>
       </c>
       <c r="J48" s="3" t="n">
+        <v>1.985327173271861</v>
+      </c>
+      <c r="K48" s="3" t="n">
+        <v>1.980093018301692</v>
+      </c>
+      <c r="L48" s="3" t="n">
+        <v>1.997926884557323</v>
+      </c>
+      <c r="M48" s="3" t="n">
+        <v>1.974928543758819</v>
+      </c>
+      <c r="N48" s="3" t="n">
+        <v>1.985257869808233</v>
+      </c>
+      <c r="O48" s="3" t="n">
+        <v>1.997549314493211</v>
+      </c>
+      <c r="P48" s="3" t="n">
+        <v>2.000736572916129</v>
+      </c>
+      <c r="Q48" s="3" t="n">
+        <v>1.989335820103864</v>
+      </c>
+      <c r="R48" s="3" t="n">
+        <v>17.56990628317934</v>
+      </c>
+      <c r="S48" s="3" t="n">
         <v>21.57855311518242</v>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="T48" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2278,15 +3601,42 @@
         <v>1.756972179821997</v>
       </c>
       <c r="H49" s="3" t="n">
-        <v>1.743135090866648</v>
+        <v>1.733396166327641</v>
       </c>
       <c r="I49" s="3" t="n">
-        <v>-0.187366960728852</v>
+        <v>1.736525345877352</v>
       </c>
       <c r="J49" s="3" t="n">
+        <v>1.738313809301958</v>
+      </c>
+      <c r="K49" s="3" t="n">
+        <v>1.736042889204407</v>
+      </c>
+      <c r="L49" s="3" t="n">
+        <v>1.737444301198309</v>
+      </c>
+      <c r="M49" s="3" t="n">
+        <v>1.735365594030607</v>
+      </c>
+      <c r="N49" s="3" t="n">
+        <v>1.729773734542677</v>
+      </c>
+      <c r="O49" s="3" t="n">
+        <v>1.762656941471223</v>
+      </c>
+      <c r="P49" s="3" t="n">
+        <v>1.746980484869774</v>
+      </c>
+      <c r="Q49" s="3" t="n">
+        <v>1.740492044951991</v>
+      </c>
+      <c r="R49" s="3" t="n">
+        <v>2.455678953928064</v>
+      </c>
+      <c r="S49" s="3" t="n">
         <v>6.422378028566378</v>
       </c>
-      <c r="K49" s="2" t="n">
+      <c r="T49" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2315,15 +3665,42 @@
         <v>2.915180599343953</v>
       </c>
       <c r="H50" s="3" t="n">
-        <v>2.908000806866664</v>
+        <v>2.913395820912104</v>
       </c>
       <c r="I50" s="3" t="n">
-        <v>6.913577685889738</v>
+        <v>2.915512142242827</v>
       </c>
       <c r="J50" s="3" t="n">
+        <v>2.914914384552554</v>
+      </c>
+      <c r="K50" s="3" t="n">
+        <v>2.912097329205084</v>
+      </c>
+      <c r="L50" s="3" t="n">
+        <v>2.918332530036758</v>
+      </c>
+      <c r="M50" s="3" t="n">
+        <v>2.915512142242827</v>
+      </c>
+      <c r="N50" s="3" t="n">
+        <v>2.91110019109039</v>
+      </c>
+      <c r="O50" s="3" t="n">
+        <v>2.915512142242827</v>
+      </c>
+      <c r="P50" s="3" t="n">
+        <v>2.913504565989889</v>
+      </c>
+      <c r="Q50" s="3" t="n">
+        <v>2.912823639092938</v>
+      </c>
+      <c r="R50" s="3" t="n">
+        <v>2.090745459616183</v>
+      </c>
+      <c r="S50" s="3" t="n">
         <v>-0.5977576902731485</v>
       </c>
-      <c r="K50" s="2" t="n">
+      <c r="T50" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2352,15 +3729,42 @@
         <v>2.725205974076549</v>
       </c>
       <c r="H51" s="3" t="n">
-        <v>2.723167984288155</v>
+        <v>2.711298741668581</v>
       </c>
       <c r="I51" s="3" t="n">
-        <v>-28.04453806299501</v>
+        <v>2.710803488663657</v>
       </c>
       <c r="J51" s="3" t="n">
+        <v>2.715359953961394</v>
+      </c>
+      <c r="K51" s="3" t="n">
+        <v>2.719418197627512</v>
+      </c>
+      <c r="L51" s="3" t="n">
+        <v>2.694863384729428</v>
+      </c>
+      <c r="M51" s="3" t="n">
+        <v>2.738927399232177</v>
+      </c>
+      <c r="N51" s="3" t="n">
+        <v>2.697635300671744</v>
+      </c>
+      <c r="O51" s="3" t="n">
+        <v>2.715077023542813</v>
+      </c>
+      <c r="P51" s="3" t="n">
+        <v>2.710430969234906</v>
+      </c>
+      <c r="Q51" s="3" t="n">
+        <v>2.715276534349723</v>
+      </c>
+      <c r="R51" s="3" t="n">
+        <v>-20.15308812456285</v>
+      </c>
+      <c r="S51" s="3" t="n">
         <v>-20.23650773623453</v>
       </c>
-      <c r="K51" s="2" t="n">
+      <c r="T51" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2389,15 +3793,42 @@
         <v>2.810719814419394</v>
       </c>
       <c r="H52" s="3" t="n">
-        <v>2.821454608740026</v>
+        <v>2.824939970230641</v>
       </c>
       <c r="I52" s="3" t="n">
-        <v>-4.925934830115164</v>
+        <v>2.832604252926104</v>
       </c>
       <c r="J52" s="3" t="n">
+        <v>2.825721044640959</v>
+      </c>
+      <c r="K52" s="3" t="n">
+        <v>2.833231732676153</v>
+      </c>
+      <c r="L52" s="3" t="n">
+        <v>2.823773003728367</v>
+      </c>
+      <c r="M52" s="3" t="n">
+        <v>2.826837777484337</v>
+      </c>
+      <c r="N52" s="3" t="n">
+        <v>2.812247541434324</v>
+      </c>
+      <c r="O52" s="3" t="n">
+        <v>2.828832594098498</v>
+      </c>
+      <c r="P52" s="3" t="n">
+        <v>2.824043525621188</v>
+      </c>
+      <c r="Q52" s="3" t="n">
+        <v>2.824716272421721</v>
+      </c>
+      <c r="R52" s="3" t="n">
+        <v>-8.187598511809835</v>
+      </c>
+      <c r="S52" s="3" t="n">
         <v>-10.30911129854406</v>
       </c>
-      <c r="K52" s="2" t="n">
+      <c r="T52" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2426,15 +3857,42 @@
         <v>2.209534965266479</v>
       </c>
       <c r="H53" s="3" t="n">
-        <v>2.221930913468174</v>
+        <v>2.188182154575627</v>
       </c>
       <c r="I53" s="3" t="n">
-        <v>192.266776704944</v>
+        <v>2.155223097489986</v>
       </c>
       <c r="J53" s="3" t="n">
+        <v>2.226705148816709</v>
+      </c>
+      <c r="K53" s="3" t="n">
+        <v>2.221370334216528</v>
+      </c>
+      <c r="L53" s="3" t="n">
+        <v>2.237904827573966</v>
+      </c>
+      <c r="M53" s="3" t="n">
+        <v>2.169618301126698</v>
+      </c>
+      <c r="N53" s="3" t="n">
+        <v>2.271057912326893</v>
+      </c>
+      <c r="O53" s="3" t="n">
+        <v>2.166230245401822</v>
+      </c>
+      <c r="P53" s="3" t="n">
+        <v>2.168231342683531</v>
+      </c>
+      <c r="Q53" s="3" t="n">
+        <v>2.20585967538469</v>
+      </c>
+      <c r="R53" s="3" t="n">
+        <v>208.3380147884282</v>
+      </c>
+      <c r="S53" s="3" t="n">
         <v>228.1192859324133</v>
       </c>
-      <c r="K53" s="2" t="n">
+      <c r="T53" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2463,15 +3921,42 @@
         <v>2.689392462825915</v>
       </c>
       <c r="H54" s="3" t="n">
-        <v>2.688274693169214</v>
+        <v>2.704795484658584</v>
       </c>
       <c r="I54" s="3" t="n">
-        <v>17.12325044933838</v>
+        <v>2.686786945917459</v>
       </c>
       <c r="J54" s="3" t="n">
+        <v>2.666782093455884</v>
+      </c>
+      <c r="K54" s="3" t="n">
+        <v>2.692817552709287</v>
+      </c>
+      <c r="L54" s="3" t="n">
+        <v>2.690892793017231</v>
+      </c>
+      <c r="M54" s="3" t="n">
+        <v>2.696260899102209</v>
+      </c>
+      <c r="N54" s="3" t="n">
+        <v>2.68965093551224</v>
+      </c>
+      <c r="O54" s="3" t="n">
+        <v>2.687966882010132</v>
+      </c>
+      <c r="P54" s="3" t="n">
+        <v>2.685108177829696</v>
+      </c>
+      <c r="Q54" s="3" t="n">
+        <v>2.688823820310031</v>
+      </c>
+      <c r="R54" s="3" t="n">
+        <v>16.57412330852193</v>
+      </c>
+      <c r="S54" s="3" t="n">
         <v>15.50394375011699</v>
       </c>
-      <c r="K54" s="2" t="n">
+      <c r="T54" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2500,15 +3985,42 @@
         <v>2.842810291228262</v>
       </c>
       <c r="H55" s="3" t="n">
-        <v>2.841994780203974</v>
+        <v>2.866551023862328</v>
       </c>
       <c r="I55" s="3" t="n">
-        <v>106.1247817373423</v>
+        <v>2.891944448414661</v>
       </c>
       <c r="J55" s="3" t="n">
+        <v>2.868138460723446</v>
+      </c>
+      <c r="K55" s="3" t="n">
+        <v>2.84280330455493</v>
+      </c>
+      <c r="L55" s="3" t="n">
+        <v>2.960089898995793</v>
+      </c>
+      <c r="M55" s="3" t="n">
+        <v>3.001900767870128</v>
+      </c>
+      <c r="N55" s="3" t="n">
+        <v>2.846104801455228</v>
+      </c>
+      <c r="O55" s="3" t="n">
+        <v>2.898459040774497</v>
+      </c>
+      <c r="P55" s="3" t="n">
+        <v>2.871630754213157</v>
+      </c>
+      <c r="Q55" s="3" t="n">
+        <v>2.881133903456341</v>
+      </c>
+      <c r="R55" s="3" t="n">
+        <v>66.98565848497529</v>
+      </c>
+      <c r="S55" s="3" t="n">
         <v>105.3162573863862</v>
       </c>
-      <c r="K55" s="2" t="n">
+      <c r="T55" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2537,15 +4049,42 @@
         <v>3.238435520412176</v>
       </c>
       <c r="H56" s="3" t="n">
-        <v>3.237302808902271</v>
+        <v>3.241305416319967</v>
       </c>
       <c r="I56" s="3" t="n">
-        <v>11.66527925967298</v>
+        <v>3.251137712344431</v>
       </c>
       <c r="J56" s="3" t="n">
+        <v>3.243764739724833</v>
+      </c>
+      <c r="K56" s="3" t="n">
+        <v>3.241320427435269</v>
+      </c>
+      <c r="L56" s="3" t="n">
+        <v>3.242679156699169</v>
+      </c>
+      <c r="M56" s="3" t="n">
+        <v>3.241797448842546</v>
+      </c>
+      <c r="N56" s="3" t="n">
+        <v>3.244243884617841</v>
+      </c>
+      <c r="O56" s="3" t="n">
+        <v>3.241808756198851</v>
+      </c>
+      <c r="P56" s="3" t="n">
+        <v>3.244402142667703</v>
+      </c>
+      <c r="Q56" s="3" t="n">
+        <v>3.242030675963118</v>
+      </c>
+      <c r="R56" s="3" t="n">
+        <v>6.937412198825488</v>
+      </c>
+      <c r="S56" s="3" t="n">
         <v>4.382788250414826</v>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="T56" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2574,15 +4113,42 @@
         <v>2.773669791307436</v>
       </c>
       <c r="H57" s="3" t="n">
-        <v>2.769138561337714</v>
+        <v>2.764190607588807</v>
       </c>
       <c r="I57" s="3" t="n">
-        <v>10.54461375823301</v>
+        <v>2.762976378571776</v>
       </c>
       <c r="J57" s="3" t="n">
+        <v>2.768341852259962</v>
+      </c>
+      <c r="K57" s="3" t="n">
+        <v>2.765712384263853</v>
+      </c>
+      <c r="L57" s="3" t="n">
+        <v>2.768135372141981</v>
+      </c>
+      <c r="M57" s="3" t="n">
+        <v>2.771717097616745</v>
+      </c>
+      <c r="N57" s="3" t="n">
+        <v>2.773467289903104</v>
+      </c>
+      <c r="O57" s="3" t="n">
+        <v>2.769096411234089</v>
+      </c>
+      <c r="P57" s="3" t="n">
+        <v>2.767768649903356</v>
+      </c>
+      <c r="Q57" s="3" t="n">
+        <v>2.768235143958067</v>
+      </c>
+      <c r="R57" s="3" t="n">
+        <v>11.44803113787951</v>
+      </c>
+      <c r="S57" s="3" t="n">
         <v>7.600453795413742</v>
       </c>
-      <c r="K57" s="2" t="n">
+      <c r="T57" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2611,15 +4177,42 @@
         <v>2.188264031519104</v>
       </c>
       <c r="H58" s="3" t="n">
-        <v>2.186885430533823</v>
+        <v>2.188277022906661</v>
       </c>
       <c r="I58" s="3" t="n">
-        <v>7.006190172181181</v>
+        <v>2.177486661694447</v>
       </c>
       <c r="J58" s="3" t="n">
+        <v>2.191914568570077</v>
+      </c>
+      <c r="K58" s="3" t="n">
+        <v>2.188952918626426</v>
+      </c>
+      <c r="L58" s="3" t="n">
+        <v>2.185989759513311</v>
+      </c>
+      <c r="M58" s="3" t="n">
+        <v>2.183578701990963</v>
+      </c>
+      <c r="N58" s="3" t="n">
+        <v>2.188376742915048</v>
+      </c>
+      <c r="O58" s="3" t="n">
+        <v>2.183962930982073</v>
+      </c>
+      <c r="P58" s="3" t="n">
+        <v>2.191357414375235</v>
+      </c>
+      <c r="Q58" s="3" t="n">
+        <v>2.186712751097976</v>
+      </c>
+      <c r="R58" s="3" t="n">
+        <v>7.178869608028382</v>
+      </c>
+      <c r="S58" s="3" t="n">
         <v>2.224646300157396</v>
       </c>
-      <c r="K58" s="2" t="n">
+      <c r="T58" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2648,15 +4241,42 @@
         <v>0.7953419074727968</v>
       </c>
       <c r="H59" s="3" t="n">
-        <v>0.7970314813590175</v>
+        <v>0.7916469321667283</v>
       </c>
       <c r="I59" s="3" t="n">
-        <v>7.559373829919447</v>
+        <v>0.7948800176001203</v>
       </c>
       <c r="J59" s="3" t="n">
+        <v>0.7932039824364759</v>
+      </c>
+      <c r="K59" s="3" t="n">
+        <v>0.7886016685662505</v>
+      </c>
+      <c r="L59" s="3" t="n">
+        <v>0.7864451010787402</v>
+      </c>
+      <c r="M59" s="3" t="n">
+        <v>0.7983208591410296</v>
+      </c>
+      <c r="N59" s="3" t="n">
+        <v>0.7917292267951972</v>
+      </c>
+      <c r="O59" s="3" t="n">
+        <v>0.79206888453442</v>
+      </c>
+      <c r="P59" s="3" t="n">
+        <v>0.7917637705621667</v>
+      </c>
+      <c r="Q59" s="3" t="n">
+        <v>0.793312907246515</v>
+      </c>
+      <c r="R59" s="3" t="n">
+        <v>11.27794794242187</v>
+      </c>
+      <c r="S59" s="3" t="n">
         <v>12.87037635724564</v>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="T59" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2685,15 +4305,42 @@
         <v>2.877264769421468</v>
       </c>
       <c r="H60" s="3" t="n">
-        <v>2.877005647173569</v>
+        <v>2.877480596201091</v>
       </c>
       <c r="I60" s="3" t="n">
-        <v>17.37988823020942</v>
+        <v>2.876880897234686</v>
       </c>
       <c r="J60" s="3" t="n">
+        <v>2.876856259653202</v>
+      </c>
+      <c r="K60" s="3" t="n">
+        <v>2.876867390792461</v>
+      </c>
+      <c r="L60" s="3" t="n">
+        <v>2.876880897234686</v>
+      </c>
+      <c r="M60" s="3" t="n">
+        <v>2.87684675412204</v>
+      </c>
+      <c r="N60" s="3" t="n">
+        <v>2.876501653892826</v>
+      </c>
+      <c r="O60" s="3" t="n">
+        <v>2.876851907895149</v>
+      </c>
+      <c r="P60" s="3" t="n">
+        <v>2.875871181684755</v>
+      </c>
+      <c r="Q60" s="3" t="n">
+        <v>2.876837873352633</v>
+      </c>
+      <c r="R60" s="3" t="n">
+        <v>17.54766205114455</v>
+      </c>
+      <c r="S60" s="3" t="n">
         <v>17.50463816909154</v>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="T60" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2722,15 +4369,42 @@
         <v>2.537028590936704</v>
       </c>
       <c r="H61" s="3" t="n">
-        <v>2.538198707952044</v>
+        <v>2.531515946178987</v>
       </c>
       <c r="I61" s="3" t="n">
-        <v>4.200607397532252</v>
+        <v>2.537093421001552</v>
       </c>
       <c r="J61" s="3" t="n">
+        <v>2.537138665839603</v>
+      </c>
+      <c r="K61" s="3" t="n">
+        <v>2.535699797194506</v>
+      </c>
+      <c r="L61" s="3" t="n">
+        <v>2.537148623968505</v>
+      </c>
+      <c r="M61" s="3" t="n">
+        <v>2.539847829353563</v>
+      </c>
+      <c r="N61" s="3" t="n">
+        <v>2.548188990367602</v>
+      </c>
+      <c r="O61" s="3" t="n">
+        <v>2.536147688489902</v>
+      </c>
+      <c r="P61" s="3" t="n">
+        <v>2.526680084975448</v>
+      </c>
+      <c r="Q61" s="3" t="n">
+        <v>2.537004764268817</v>
+      </c>
+      <c r="R61" s="3" t="n">
+        <v>5.394551080759147</v>
+      </c>
+      <c r="S61" s="3" t="n">
         <v>5.250691159220278</v>
       </c>
-      <c r="K61" s="2" t="n">
+      <c r="T61" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2759,15 +4433,42 @@
         <v>2.364785825017967</v>
       </c>
       <c r="H62" s="3" t="n">
-        <v>2.372077256447291</v>
+        <v>2.385698078147262</v>
       </c>
       <c r="I62" s="3" t="n">
-        <v>-1.206223722056254</v>
+        <v>2.369625307408365</v>
       </c>
       <c r="J62" s="3" t="n">
+        <v>2.362693861266005</v>
+      </c>
+      <c r="K62" s="3" t="n">
+        <v>2.364481352817825</v>
+      </c>
+      <c r="L62" s="3" t="n">
+        <v>2.343830367205941</v>
+      </c>
+      <c r="M62" s="3" t="n">
+        <v>2.363959729024907</v>
+      </c>
+      <c r="N62" s="3" t="n">
+        <v>2.36429775697178</v>
+      </c>
+      <c r="O62" s="3" t="n">
+        <v>2.307937579012531</v>
+      </c>
+      <c r="P62" s="3" t="n">
+        <v>2.369285470826238</v>
+      </c>
+      <c r="Q62" s="3" t="n">
+        <v>2.362336772668561</v>
+      </c>
+      <c r="R62" s="3" t="n">
+        <v>8.53426005667357</v>
+      </c>
+      <c r="S62" s="3" t="n">
         <v>6.598458463233037</v>
       </c>
-      <c r="K62" s="2" t="n">
+      <c r="T62" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2796,15 +4497,42 @@
         <v>2.384490190826773</v>
       </c>
       <c r="H63" s="3" t="n">
-        <v>2.384041626891767</v>
+        <v>2.393660275040383</v>
       </c>
       <c r="I63" s="3" t="n">
-        <v>-1.141146332716669</v>
+        <v>2.359397004795164</v>
       </c>
       <c r="J63" s="3" t="n">
+        <v>2.382847442057655</v>
+      </c>
+      <c r="K63" s="3" t="n">
+        <v>2.384661034725906</v>
+      </c>
+      <c r="L63" s="3" t="n">
+        <v>2.392743650381504</v>
+      </c>
+      <c r="M63" s="3" t="n">
+        <v>2.376068992396659</v>
+      </c>
+      <c r="N63" s="3" t="n">
+        <v>2.383001737182164</v>
+      </c>
+      <c r="O63" s="3" t="n">
+        <v>2.376236748419233</v>
+      </c>
+      <c r="P63" s="3" t="n">
+        <v>2.38169875584917</v>
+      </c>
+      <c r="Q63" s="3" t="n">
+        <v>2.381870043460262</v>
+      </c>
+      <c r="R63" s="3" t="n">
+        <v>1.030437098788806</v>
+      </c>
+      <c r="S63" s="3" t="n">
         <v>-2.118684959596884</v>
       </c>
-      <c r="K63" s="2" t="n">
+      <c r="T63" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2833,15 +4561,42 @@
         <v>2.161317904763674</v>
       </c>
       <c r="H64" s="3" t="n">
-        <v>2.155807077976332</v>
+        <v>2.168894371211752</v>
       </c>
       <c r="I64" s="3" t="n">
-        <v>13.3382974744527</v>
+        <v>2.169067138831105</v>
       </c>
       <c r="J64" s="3" t="n">
+        <v>2.170604912069827</v>
+      </c>
+      <c r="K64" s="3" t="n">
+        <v>2.16989702277391</v>
+      </c>
+      <c r="L64" s="3" t="n">
+        <v>2.170194219397088</v>
+      </c>
+      <c r="M64" s="3" t="n">
+        <v>2.16862337968111</v>
+      </c>
+      <c r="N64" s="3" t="n">
+        <v>2.169148376900663</v>
+      </c>
+      <c r="O64" s="3" t="n">
+        <v>2.178609011049423</v>
+      </c>
+      <c r="P64" s="3" t="n">
+        <v>2.169184084875396</v>
+      </c>
+      <c r="Q64" s="3" t="n">
+        <v>2.166803645893273</v>
+      </c>
+      <c r="R64" s="3" t="n">
+        <v>2.341729557512107</v>
+      </c>
+      <c r="S64" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K64" s="2" t="n">
+      <c r="T64" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2870,15 +4625,42 @@
         <v>2.282945280269624</v>
       </c>
       <c r="H65" s="3" t="n">
-        <v>2.282894875202557</v>
+        <v>2.282110629798264</v>
       </c>
       <c r="I65" s="3" t="n">
-        <v>7.761966339439486</v>
+        <v>2.282930718681359</v>
       </c>
       <c r="J65" s="3" t="n">
+        <v>2.28239637096877</v>
+      </c>
+      <c r="K65" s="3" t="n">
+        <v>2.283016083703931</v>
+      </c>
+      <c r="L65" s="3" t="n">
+        <v>2.283144865580599</v>
+      </c>
+      <c r="M65" s="3" t="n">
+        <v>2.281650425517899</v>
+      </c>
+      <c r="N65" s="3" t="n">
+        <v>2.281684680975829</v>
+      </c>
+      <c r="O65" s="3" t="n">
+        <v>2.282515981222367</v>
+      </c>
+      <c r="P65" s="3" t="n">
+        <v>2.282806614021668</v>
+      </c>
+      <c r="Q65" s="3" t="n">
+        <v>2.282578416339863</v>
+      </c>
+      <c r="R65" s="3" t="n">
+        <v>8.07842520213331</v>
+      </c>
+      <c r="S65" s="3" t="n">
         <v>7.711549434562315</v>
       </c>
-      <c r="K65" s="2" t="n">
+      <c r="T65" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2907,15 +4689,42 @@
         <v>2.925970651457613</v>
       </c>
       <c r="H66" s="3" t="n">
-        <v>2.92600270835671</v>
+        <v>2.926325055642457</v>
       </c>
       <c r="I66" s="3" t="n">
-        <v>0.2294759423793202</v>
+        <v>2.922728251649851</v>
       </c>
       <c r="J66" s="3" t="n">
+        <v>2.920607646427051</v>
+      </c>
+      <c r="K66" s="3" t="n">
+        <v>2.926438994467668</v>
+      </c>
+      <c r="L66" s="3" t="n">
+        <v>2.92602263716825</v>
+      </c>
+      <c r="M66" s="3" t="n">
+        <v>2.926495395713403</v>
+      </c>
+      <c r="N66" s="3" t="n">
+        <v>2.923346794159384</v>
+      </c>
+      <c r="O66" s="3" t="n">
+        <v>2.922272405860586</v>
+      </c>
+      <c r="P66" s="3" t="n">
+        <v>2.926668954605984</v>
+      </c>
+      <c r="Q66" s="3" t="n">
+        <v>2.924909521730397</v>
+      </c>
+      <c r="R66" s="3" t="n">
+        <v>1.322662568692401</v>
+      </c>
+      <c r="S66" s="3" t="n">
         <v>-0.436770306894374</v>
       </c>
-      <c r="K66" s="2" t="n">
+      <c r="T66" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2944,15 +4753,42 @@
         <v>2.632621465848895</v>
       </c>
       <c r="H67" s="3" t="n">
-        <v>2.634822460416269</v>
+        <v>2.615666321723654</v>
       </c>
       <c r="I67" s="3" t="n">
-        <v>23.1573286740856</v>
+        <v>2.605879757696125</v>
       </c>
       <c r="J67" s="3" t="n">
+        <v>2.629449021698886</v>
+      </c>
+      <c r="K67" s="3" t="n">
+        <v>2.631895609604311</v>
+      </c>
+      <c r="L67" s="3" t="n">
+        <v>2.63192897344525</v>
+      </c>
+      <c r="M67" s="3" t="n">
+        <v>2.634992242325465</v>
+      </c>
+      <c r="N67" s="3" t="n">
+        <v>2.63499307764462</v>
+      </c>
+      <c r="O67" s="3" t="n">
+        <v>2.62720020194985</v>
+      </c>
+      <c r="P67" s="3" t="n">
+        <v>2.630008155934955</v>
+      </c>
+      <c r="Q67" s="3" t="n">
+        <v>2.62887339527266</v>
+      </c>
+      <c r="R67" s="3" t="n">
+        <v>29.10639381769453</v>
+      </c>
+      <c r="S67" s="3" t="n">
         <v>22.98671144573428</v>
       </c>
-      <c r="K67" s="2" t="n">
+      <c r="T67" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2981,15 +4817,42 @@
         <v>2.876598790812057</v>
       </c>
       <c r="H68" s="3" t="n">
-        <v>2.877383932972657</v>
+        <v>2.873144284249785</v>
       </c>
       <c r="I68" s="3" t="n">
-        <v>6.837544272222829</v>
+        <v>2.877834233821817</v>
       </c>
       <c r="J68" s="3" t="n">
+        <v>2.854630510081289</v>
+      </c>
+      <c r="K68" s="3" t="n">
+        <v>2.868963229366371</v>
+      </c>
+      <c r="L68" s="3" t="n">
+        <v>2.872331689609156</v>
+      </c>
+      <c r="M68" s="3" t="n">
+        <v>2.871136383985604</v>
+      </c>
+      <c r="N68" s="3" t="n">
+        <v>2.881920654971128</v>
+      </c>
+      <c r="O68" s="3" t="n">
+        <v>2.873964316103902</v>
+      </c>
+      <c r="P68" s="3" t="n">
+        <v>2.877989609073832</v>
+      </c>
+      <c r="Q68" s="3" t="n">
+        <v>2.873672225848404</v>
+      </c>
+      <c r="R68" s="3" t="n">
+        <v>10.54925139647578</v>
+      </c>
+      <c r="S68" s="3" t="n">
         <v>6.357205324174942</v>
       </c>
-      <c r="K68" s="2" t="n">
+      <c r="T68" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3018,15 +4881,42 @@
         <v>1.354314617862723</v>
       </c>
       <c r="H69" s="3" t="n">
-        <v>1.386658063416069</v>
+        <v>1.388433661209928</v>
       </c>
       <c r="I69" s="3" t="n">
-        <v>56.53001770659438</v>
+        <v>1.410281897272516</v>
       </c>
       <c r="J69" s="3" t="n">
+        <v>1.379069712144466</v>
+      </c>
+      <c r="K69" s="3" t="n">
+        <v>1.389024145205726</v>
+      </c>
+      <c r="L69" s="3" t="n">
+        <v>1.397132971403206</v>
+      </c>
+      <c r="M69" s="3" t="n">
+        <v>1.35417097312235</v>
+      </c>
+      <c r="N69" s="3" t="n">
+        <v>1.393866320195821</v>
+      </c>
+      <c r="O69" s="3" t="n">
+        <v>1.386632850577785</v>
+      </c>
+      <c r="P69" s="3" t="n">
+        <v>1.396983029315566</v>
+      </c>
+      <c r="Q69" s="3" t="n">
+        <v>1.387964145891297</v>
+      </c>
+      <c r="R69" s="3" t="n">
+        <v>55.22393523136549</v>
+      </c>
+      <c r="S69" s="3" t="n">
         <v>88.8734632599395</v>
       </c>
-      <c r="K69" s="2" t="n">
+      <c r="T69" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3055,15 +4945,42 @@
         <v>2.876960134139686</v>
       </c>
       <c r="H70" s="3" t="n">
-        <v>2.877263657300474</v>
+        <v>2.864553763297639</v>
       </c>
       <c r="I70" s="3" t="n">
-        <v>40.3564500031961</v>
+        <v>2.893845296894213</v>
       </c>
       <c r="J70" s="3" t="n">
+        <v>2.892993726822732</v>
+      </c>
+      <c r="K70" s="3" t="n">
+        <v>2.876042803822406</v>
+      </c>
+      <c r="L70" s="3" t="n">
+        <v>2.876174399569818</v>
+      </c>
+      <c r="M70" s="3" t="n">
+        <v>2.875121316166513</v>
+      </c>
+      <c r="N70" s="3" t="n">
+        <v>2.86195997589334</v>
+      </c>
+      <c r="O70" s="3" t="n">
+        <v>2.879107082879874</v>
+      </c>
+      <c r="P70" s="3" t="n">
+        <v>2.861651128207261</v>
+      </c>
+      <c r="Q70" s="3" t="n">
+        <v>2.876103372121268</v>
+      </c>
+      <c r="R70" s="3" t="n">
+        <v>41.51673518240217</v>
+      </c>
+      <c r="S70" s="3" t="n">
         <v>41.93344853803982</v>
       </c>
-      <c r="K70" s="2" t="n">
+      <c r="T70" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3092,15 +5009,42 @@
         <v>2.600391290543495</v>
       </c>
       <c r="H71" s="3" t="n">
-        <v>2.597188175145102</v>
+        <v>2.59847927026087</v>
       </c>
       <c r="I71" s="3" t="n">
-        <v>1.908938489072032</v>
+        <v>2.595046002191781</v>
       </c>
       <c r="J71" s="3" t="n">
+        <v>2.570867480694923</v>
+      </c>
+      <c r="K71" s="3" t="n">
+        <v>2.597158190147189</v>
+      </c>
+      <c r="L71" s="3" t="n">
+        <v>2.592845038592202</v>
+      </c>
+      <c r="M71" s="3" t="n">
+        <v>2.600608725972048</v>
+      </c>
+      <c r="N71" s="3" t="n">
+        <v>2.603497704298902</v>
+      </c>
+      <c r="O71" s="3" t="n">
+        <v>2.595408575869918</v>
+      </c>
+      <c r="P71" s="3" t="n">
+        <v>2.599154717672308</v>
+      </c>
+      <c r="Q71" s="3" t="n">
+        <v>2.595385852594621</v>
+      </c>
+      <c r="R71" s="3" t="n">
+        <v>3.711261039553992</v>
+      </c>
+      <c r="S71" s="3" t="n">
         <v>-1.510239920332612</v>
       </c>
-      <c r="K71" s="2" t="n">
+      <c r="T71" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3129,15 +5073,42 @@
         <v>2.290922464481045</v>
       </c>
       <c r="H72" s="3" t="n">
-        <v>2.301283065507839</v>
+        <v>2.30607171827633</v>
       </c>
       <c r="I72" s="3" t="n">
-        <v>58.45059328449675</v>
+        <v>2.300877039754242</v>
       </c>
       <c r="J72" s="3" t="n">
+        <v>2.306137954752097</v>
+      </c>
+      <c r="K72" s="3" t="n">
+        <v>2.321658949692006</v>
+      </c>
+      <c r="L72" s="3" t="n">
+        <v>2.297798783615746</v>
+      </c>
+      <c r="M72" s="3" t="n">
+        <v>2.304416540142063</v>
+      </c>
+      <c r="N72" s="3" t="n">
+        <v>2.305088835448111</v>
+      </c>
+      <c r="O72" s="3" t="n">
+        <v>2.294652278808146</v>
+      </c>
+      <c r="P72" s="3" t="n">
+        <v>2.322804171641313</v>
+      </c>
+      <c r="Q72" s="3" t="n">
+        <v>2.305279622387797</v>
+      </c>
+      <c r="R72" s="3" t="n">
+        <v>54.45403640453827</v>
+      </c>
+      <c r="S72" s="3" t="n">
         <v>53.59570258213786</v>
       </c>
-      <c r="K72" s="2" t="n">
+      <c r="T72" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3166,15 +5137,42 @@
         <v>2.776820041659729</v>
       </c>
       <c r="H73" s="3" t="n">
-        <v>2.776371716199137</v>
+        <v>2.77586037643097</v>
       </c>
       <c r="I73" s="3" t="n">
-        <v>-2.727173198834087</v>
+        <v>2.759004796472259</v>
       </c>
       <c r="J73" s="3" t="n">
+        <v>2.774488603770713</v>
+      </c>
+      <c r="K73" s="3" t="n">
+        <v>2.775853341601584</v>
+      </c>
+      <c r="L73" s="3" t="n">
+        <v>2.776982694940489</v>
+      </c>
+      <c r="M73" s="3" t="n">
+        <v>2.775562853838838</v>
+      </c>
+      <c r="N73" s="3" t="n">
+        <v>2.776214901441297</v>
+      </c>
+      <c r="O73" s="3" t="n">
+        <v>2.773877160401074</v>
+      </c>
+      <c r="P73" s="3" t="n">
+        <v>2.775975537664318</v>
+      </c>
+      <c r="Q73" s="3" t="n">
+        <v>2.774411284596579</v>
+      </c>
+      <c r="R73" s="3" t="n">
+        <v>-0.7667415962768764</v>
+      </c>
+      <c r="S73" s="3" t="n">
         <v>-2.524651664463473</v>
       </c>
-      <c r="K73" s="2" t="n">
+      <c r="T73" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3203,15 +5201,42 @@
         <v>2.492039810245472</v>
       </c>
       <c r="H74" s="3" t="n">
-        <v>2.479426123379261</v>
+        <v>2.446266831771855</v>
       </c>
       <c r="I74" s="3" t="n">
-        <v>25.28768300479145</v>
+        <v>2.455984543877225</v>
       </c>
       <c r="J74" s="3" t="n">
+        <v>2.486218509485236</v>
+      </c>
+      <c r="K74" s="3" t="n">
+        <v>2.45925082079586</v>
+      </c>
+      <c r="L74" s="3" t="n">
+        <v>2.460481096926892</v>
+      </c>
+      <c r="M74" s="3" t="n">
+        <v>2.459052277985313</v>
+      </c>
+      <c r="N74" s="3" t="n">
+        <v>2.504484430816661</v>
+      </c>
+      <c r="O74" s="3" t="n">
+        <v>2.459779648010658</v>
+      </c>
+      <c r="P74" s="3" t="n">
+        <v>2.450524773165207</v>
+      </c>
+      <c r="Q74" s="3" t="n">
+        <v>2.468360108581058</v>
+      </c>
+      <c r="R74" s="3" t="n">
+        <v>36.35369780299502</v>
+      </c>
+      <c r="S74" s="3" t="n">
         <v>44.23270888630304</v>
       </c>
-      <c r="K74" s="2" t="n">
+      <c r="T74" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3240,15 +5265,42 @@
         <v>2.815505944330686</v>
       </c>
       <c r="H75" s="3" t="n">
-        <v>2.815752102241503</v>
+        <v>2.815485940684587</v>
       </c>
       <c r="I75" s="3" t="n">
-        <v>-17.73497991112238</v>
+        <v>2.814494883989545</v>
       </c>
       <c r="J75" s="3" t="n">
+        <v>2.816685843628303</v>
+      </c>
+      <c r="K75" s="3" t="n">
+        <v>2.823237072131115</v>
+      </c>
+      <c r="L75" s="3" t="n">
+        <v>2.811772539592289</v>
+      </c>
+      <c r="M75" s="3" t="n">
+        <v>2.823461581748718</v>
+      </c>
+      <c r="N75" s="3" t="n">
+        <v>2.812139209399509</v>
+      </c>
+      <c r="O75" s="3" t="n">
+        <v>2.815396085205334</v>
+      </c>
+      <c r="P75" s="3" t="n">
+        <v>2.800897599447256</v>
+      </c>
+      <c r="Q75" s="3" t="n">
+        <v>2.815068921879263</v>
+      </c>
+      <c r="R75" s="3" t="n">
+        <v>-17.05179954888303</v>
+      </c>
+      <c r="S75" s="3" t="n">
         <v>-17.51103748292593</v>
       </c>
-      <c r="K75" s="2" t="n">
+      <c r="T75" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3277,15 +5329,42 @@
         <v>2.476016837609721</v>
       </c>
       <c r="H76" s="3" t="n">
-        <v>2.493850313227228</v>
+        <v>2.348370929100267</v>
       </c>
       <c r="I76" s="3" t="n">
-        <v>140.0425989470615</v>
+        <v>2.595651394617729</v>
       </c>
       <c r="J76" s="3" t="n">
+        <v>2.368179791624013</v>
+      </c>
+      <c r="K76" s="3" t="n">
+        <v>2.488110093040359</v>
+      </c>
+      <c r="L76" s="3" t="n">
+        <v>2.32542747672239</v>
+      </c>
+      <c r="M76" s="3" t="n">
+        <v>2.653376444130231</v>
+      </c>
+      <c r="N76" s="3" t="n">
+        <v>2.421666266871532</v>
+      </c>
+      <c r="O76" s="3" t="n">
+        <v>2.688496763429085</v>
+      </c>
+      <c r="P76" s="3" t="n">
+        <v>2.331057749495088</v>
+      </c>
+      <c r="Q76" s="3" t="n">
+        <v>2.475157320726032</v>
+      </c>
+      <c r="R76" s="3" t="n">
+        <v>158.735591448258</v>
+      </c>
+      <c r="S76" s="3" t="n">
         <v>307.1570063906775</v>
       </c>
-      <c r="K76" s="2" t="n">
+      <c r="T76" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3314,15 +5393,42 @@
         <v>1.563802603451571</v>
       </c>
       <c r="H77" s="3" t="n">
-        <v>1.570477852693911</v>
+        <v>1.562135601925865</v>
       </c>
       <c r="I77" s="3" t="n">
-        <v>104.0733354589101</v>
+        <v>1.560665864358825</v>
       </c>
       <c r="J77" s="3" t="n">
+        <v>1.606386389267433</v>
+      </c>
+      <c r="K77" s="3" t="n">
+        <v>1.562323475499729</v>
+      </c>
+      <c r="L77" s="3" t="n">
+        <v>1.559011123363683</v>
+      </c>
+      <c r="M77" s="3" t="n">
+        <v>1.55496692710049</v>
+      </c>
+      <c r="N77" s="3" t="n">
+        <v>1.582580205637495</v>
+      </c>
+      <c r="O77" s="3" t="n">
+        <v>1.567132788842478</v>
+      </c>
+      <c r="P77" s="3" t="n">
+        <v>1.562113644989008</v>
+      </c>
+      <c r="Q77" s="3" t="n">
+        <v>1.569062464922228</v>
+      </c>
+      <c r="R77" s="3" t="n">
+        <v>105.488723230593</v>
+      </c>
+      <c r="S77" s="3" t="n">
         <v>112.2277126530928</v>
       </c>
-      <c r="K77" s="2" t="n">
+      <c r="T77" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3351,15 +5457,42 @@
         <v>2.442114393442605</v>
       </c>
       <c r="H78" s="3" t="n">
-        <v>2.443853422705</v>
+        <v>2.450576894202877</v>
       </c>
       <c r="I78" s="3" t="n">
-        <v>12.1754899687212</v>
+        <v>2.443683980191888</v>
       </c>
       <c r="J78" s="3" t="n">
+        <v>2.438054135633111</v>
+      </c>
+      <c r="K78" s="3" t="n">
+        <v>2.443926380754753</v>
+      </c>
+      <c r="L78" s="3" t="n">
+        <v>2.442526162326523</v>
+      </c>
+      <c r="M78" s="3" t="n">
+        <v>2.443290978300204</v>
+      </c>
+      <c r="N78" s="3" t="n">
+        <v>2.442897447909186</v>
+      </c>
+      <c r="O78" s="3" t="n">
+        <v>2.452550186666972</v>
+      </c>
+      <c r="P78" s="3" t="n">
+        <v>2.443804381784147</v>
+      </c>
+      <c r="Q78" s="3" t="n">
+        <v>2.444405901323722</v>
+      </c>
+      <c r="R78" s="3" t="n">
+        <v>11.62301134999977</v>
+      </c>
+      <c r="S78" s="3" t="n">
         <v>12.06734400969633</v>
       </c>
-      <c r="K78" s="2" t="n">
+      <c r="T78" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3388,15 +5521,42 @@
         <v>2.117812112992747</v>
       </c>
       <c r="H79" s="3" t="n">
-        <v>2.11893982411567</v>
+        <v>2.104361164536275</v>
       </c>
       <c r="I79" s="3" t="n">
-        <v>0.02023964715736071</v>
+        <v>2.111910884927525</v>
       </c>
       <c r="J79" s="3" t="n">
+        <v>2.105160395742673</v>
+      </c>
+      <c r="K79" s="3" t="n">
+        <v>2.119651004540769</v>
+      </c>
+      <c r="L79" s="3" t="n">
+        <v>2.119939148525092</v>
+      </c>
+      <c r="M79" s="3" t="n">
+        <v>2.108859358948495</v>
+      </c>
+      <c r="N79" s="3" t="n">
+        <v>2.111265993560589</v>
+      </c>
+      <c r="O79" s="3" t="n">
+        <v>2.117669942412144</v>
+      </c>
+      <c r="P79" s="3" t="n">
+        <v>2.10620309271175</v>
+      </c>
+      <c r="Q79" s="3" t="n">
+        <v>2.11348670485436</v>
+      </c>
+      <c r="R79" s="3" t="n">
+        <v>5.473358908467674</v>
+      </c>
+      <c r="S79" s="3" t="n">
         <v>-0.6404200205243349</v>
       </c>
-      <c r="K79" s="2" t="n">
+      <c r="T79" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3425,15 +5585,42 @@
         <v>2.312687946266129</v>
       </c>
       <c r="H80" s="3" t="n">
-        <v>2.322888418672237</v>
+        <v>2.32735107155775</v>
       </c>
       <c r="I80" s="3" t="n">
-        <v>-50.64621523531576</v>
+        <v>2.318852667197041</v>
       </c>
       <c r="J80" s="3" t="n">
+        <v>2.329052312063999</v>
+      </c>
+      <c r="K80" s="3" t="n">
+        <v>2.321354189226233</v>
+      </c>
+      <c r="L80" s="3" t="n">
+        <v>2.327351105383869</v>
+      </c>
+      <c r="M80" s="3" t="n">
+        <v>2.315756711629024</v>
+      </c>
+      <c r="N80" s="3" t="n">
+        <v>2.324074356564803</v>
+      </c>
+      <c r="O80" s="3" t="n">
+        <v>2.329606002062797</v>
+      </c>
+      <c r="P80" s="3" t="n">
+        <v>2.323858414146029</v>
+      </c>
+      <c r="Q80" s="3" t="n">
+        <v>2.323826840487355</v>
+      </c>
+      <c r="R80" s="3" t="n">
+        <v>-51.58463705043381</v>
+      </c>
+      <c r="S80" s="3" t="n">
         <v>-57.41259588099368</v>
       </c>
-      <c r="K80" s="2" t="n">
+      <c r="T80" s="2" t="n">
         <v>0</v>
       </c>
     </row>
@@ -3462,20 +5649,47 @@
         <v>1.925970121388174</v>
       </c>
       <c r="H81" s="3" t="n">
-        <v>1.925126171665877</v>
+        <v>1.931860680879343</v>
       </c>
       <c r="I81" s="3" t="n">
-        <v>6.734509213466522</v>
+        <v>1.91416145919835</v>
       </c>
       <c r="J81" s="3" t="n">
+        <v>1.937838586230011</v>
+      </c>
+      <c r="K81" s="3" t="n">
+        <v>1.928079130252348</v>
+      </c>
+      <c r="L81" s="3" t="n">
+        <v>1.934761939565003</v>
+      </c>
+      <c r="M81" s="3" t="n">
+        <v>1.97181475897516</v>
+      </c>
+      <c r="N81" s="3" t="n">
+        <v>1.960983470901496</v>
+      </c>
+      <c r="O81" s="3" t="n">
+        <v>1.915186813357326</v>
+      </c>
+      <c r="P81" s="3" t="n">
+        <v>1.932416233286024</v>
+      </c>
+      <c r="Q81" s="3" t="n">
+        <v>1.933540132303558</v>
+      </c>
+      <c r="R81" s="3" t="n">
+        <v>-1.67945142421444</v>
+      </c>
+      <c r="S81" s="3" t="n">
         <v>0</v>
       </c>
-      <c r="K81" s="2" t="n">
+      <c r="T81" s="2" t="n">
         <v>0</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K81"/>
+  <autoFilter ref="A1:T81"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3486,7 +5700,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E8"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -3610,61 +5824,250 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Randomized mean</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>489.3333333333333</v>
+          <t>Randomized 2404</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>504</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>237.9959104227214</v>
+        <v>237.7853511257844</v>
       </c>
       <c r="D6" s="3" t="n">
-        <v>0.03257906187687354</v>
+        <v>-0.177980235060204</v>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Three seeds averaged within date</t>
+          <t>Hash-based schedule; same target and gain as ECF</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>ECF</t>
+          <t>Randomized 2405</t>
         </is>
       </c>
       <c r="B7" s="2" t="n">
-        <v>483</v>
+        <v>475</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>239.3555652630994</v>
+        <v>238.1611912070061</v>
       </c>
       <c r="D7" s="3" t="n">
-        <v>1.392233902254816</v>
+        <v>0.1978598461615775</v>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Replay-qualified update</t>
+          <t>Hash-based schedule; same target and gain as ECF</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>Randomized 2406</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>481</v>
+      </c>
+      <c r="C8" s="3" t="n">
+        <v>237.8635391091661</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>-0.09979225167842287</v>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>Hash-based schedule; same target and gain as ECF</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Randomized 2407</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>473</v>
+      </c>
+      <c r="C9" s="3" t="n">
+        <v>238.0579412451361</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>0.09460988429154327</v>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>Hash-based schedule; same target and gain as ECF</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>Randomized 2408</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>498</v>
+      </c>
+      <c r="C10" s="3" t="n">
+        <v>237.7892981259306</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>-0.1740332349139351</v>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>Hash-based schedule; same target and gain as ECF</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Randomized 2409</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>463</v>
+      </c>
+      <c r="C11" s="3" t="n">
+        <v>238.4390420637025</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>0.475710702857981</v>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>Hash-based schedule; same target and gain as ECF</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Randomized 2410</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>468</v>
+      </c>
+      <c r="C12" s="3" t="n">
+        <v>238.1444283484542</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>0.1810969876096635</v>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>Hash-based schedule; same target and gain as ECF</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>Randomized 2411</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>519</v>
+      </c>
+      <c r="C13" s="3" t="n">
+        <v>238.1595975041229</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>0.1962661432783079</v>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>Hash-based schedule; same target and gain as ECF</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Randomized 2412</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="n">
+        <v>506</v>
+      </c>
+      <c r="C14" s="3" t="n">
+        <v>237.7594056318637</v>
+      </c>
+      <c r="D14" s="3" t="n">
+        <v>-0.2039257289808916</v>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>Hash-based schedule; same target and gain as ECF</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>Randomized mean</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>487.9166666666667</v>
+      </c>
+      <c r="C15" s="3" t="n">
+        <v>238.0122938024442</v>
+      </c>
+      <c r="D15" s="3" t="n">
+        <v>0.0489624415996559</v>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>Twelve fixed seeds averaged within date</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>ECF</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="n">
+        <v>483</v>
+      </c>
+      <c r="C16" s="3" t="n">
+        <v>239.3555652630994</v>
+      </c>
+      <c r="D16" s="3" t="n">
+        <v>1.392233902254816</v>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>Replay-qualified update</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
           <t>Update every unused award</t>
         </is>
       </c>
-      <c r="B8" s="2" t="n">
+      <c r="B17" s="2" t="n">
         <v>3086</v>
       </c>
-      <c r="C8" s="3" t="n">
+      <c r="C17" s="3" t="n">
         <v>232.9328995482401</v>
       </c>
-      <c r="D8" s="3" t="n">
+      <c r="D17" s="3" t="n">
         <v>-5.030431812604462</v>
       </c>
-      <c r="E8" s="2" t="inlineStr">
+      <c r="E17" s="2" t="inlineStr">
         <is>
           <t>Same target and gain; no replay test</t>
         </is>
@@ -3689,7 +6092,7 @@
     <col width="20" customWidth="1" min="3" max="3"/>
     <col width="21" customWidth="1" min="4" max="4"/>
     <col width="21" customWidth="1" min="5" max="5"/>
-    <col width="33" customWidth="1" min="6" max="6"/>
+    <col width="34" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -3803,20 +6206,20 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>328.3135158367048</v>
+        <v>328.3570550236519</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>90.31760541398332</v>
+        <v>90.34476122120758</v>
       </c>
       <c r="D5" s="3" t="n">
-        <v>237.9959104227214</v>
+        <v>238.0122938024442</v>
       </c>
       <c r="E5" s="3" t="n">
-        <v>489.3333333333333</v>
+        <v>487.9166666666667</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Three fixed schedules averaged</t>
+          <t>Twelve fixed schedules averaged</t>
         </is>
       </c>
     </row>
@@ -3855,7 +6258,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L4"/>
+  <dimension ref="A1:L13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4046,6 +6449,348 @@
       </c>
       <c r="L4" s="2" t="n">
         <v>43628</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="n">
+        <v>2404</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>504</v>
+      </c>
+      <c r="C5" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D5" s="3" t="n">
+        <v>328.0486928882615</v>
+      </c>
+      <c r="E5" s="3" t="n">
+        <v>90.26334176247714</v>
+      </c>
+      <c r="F5" s="3" t="n">
+        <v>237.7853511257844</v>
+      </c>
+      <c r="G5" s="3" t="n">
+        <v>1.570214137315013</v>
+      </c>
+      <c r="H5" s="2" t="n">
+        <v>58</v>
+      </c>
+      <c r="I5" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L5" s="2" t="n">
+        <v>43611</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="2" t="n">
+        <v>2405</v>
+      </c>
+      <c r="B6" s="2" t="n">
+        <v>475</v>
+      </c>
+      <c r="C6" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D6" s="3" t="n">
+        <v>328.384578449597</v>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>90.22338724259086</v>
+      </c>
+      <c r="F6" s="3" t="n">
+        <v>238.1611912070061</v>
+      </c>
+      <c r="G6" s="3" t="n">
+        <v>1.194374056093225</v>
+      </c>
+      <c r="H6" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I6" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L6" s="2" t="n">
+        <v>43628</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="n">
+        <v>2406</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>481</v>
+      </c>
+      <c r="C7" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D7" s="3" t="n">
+        <v>328.3156937878097</v>
+      </c>
+      <c r="E7" s="3" t="n">
+        <v>90.45215467864351</v>
+      </c>
+      <c r="F7" s="3" t="n">
+        <v>237.8635391091661</v>
+      </c>
+      <c r="G7" s="3" t="n">
+        <v>1.492026153933247</v>
+      </c>
+      <c r="H7" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="I7" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L7" s="2" t="n">
+        <v>43611</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="n">
+        <v>2407</v>
+      </c>
+      <c r="B8" s="2" t="n">
+        <v>473</v>
+      </c>
+      <c r="C8" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D8" s="3" t="n">
+        <v>328.3352364403281</v>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>90.27729519519201</v>
+      </c>
+      <c r="F8" s="3" t="n">
+        <v>238.0579412451361</v>
+      </c>
+      <c r="G8" s="3" t="n">
+        <v>1.297624017963262</v>
+      </c>
+      <c r="H8" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="I8" s="2" t="n">
+        <v>24</v>
+      </c>
+      <c r="J8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>43611</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="n">
+        <v>2408</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>498</v>
+      </c>
+      <c r="C9" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D9" s="3" t="n">
+        <v>328.105138919784</v>
+      </c>
+      <c r="E9" s="3" t="n">
+        <v>90.31584079385334</v>
+      </c>
+      <c r="F9" s="3" t="n">
+        <v>237.7892981259306</v>
+      </c>
+      <c r="G9" s="3" t="n">
+        <v>1.566267137168747</v>
+      </c>
+      <c r="H9" s="2" t="n">
+        <v>60</v>
+      </c>
+      <c r="I9" s="2" t="n">
+        <v>20</v>
+      </c>
+      <c r="J9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L9" s="2" t="n">
+        <v>43611</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="n">
+        <v>2409</v>
+      </c>
+      <c r="B10" s="2" t="n">
+        <v>463</v>
+      </c>
+      <c r="C10" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D10" s="3" t="n">
+        <v>328.8404439290151</v>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>90.40140186531249</v>
+      </c>
+      <c r="F10" s="3" t="n">
+        <v>238.4390420637025</v>
+      </c>
+      <c r="G10" s="3" t="n">
+        <v>0.9165231993968228</v>
+      </c>
+      <c r="H10" s="2" t="n">
+        <v>51</v>
+      </c>
+      <c r="I10" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="J10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>43628</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="n">
+        <v>2410</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>468</v>
+      </c>
+      <c r="C11" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D11" s="3" t="n">
+        <v>328.5447559596842</v>
+      </c>
+      <c r="E11" s="3" t="n">
+        <v>90.40032761122994</v>
+      </c>
+      <c r="F11" s="3" t="n">
+        <v>238.1444283484542</v>
+      </c>
+      <c r="G11" s="3" t="n">
+        <v>1.211136914645164</v>
+      </c>
+      <c r="H11" s="2" t="n">
+        <v>57</v>
+      </c>
+      <c r="I11" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="J11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>43628</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n">
+        <v>2411</v>
+      </c>
+      <c r="B12" s="2" t="n">
+        <v>519</v>
+      </c>
+      <c r="C12" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D12" s="3" t="n">
+        <v>328.6985200052853</v>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>90.53892250116238</v>
+      </c>
+      <c r="F12" s="3" t="n">
+        <v>238.1595975041229</v>
+      </c>
+      <c r="G12" s="3" t="n">
+        <v>1.195967758976493</v>
+      </c>
+      <c r="H12" s="2" t="n">
+        <v>59</v>
+      </c>
+      <c r="I12" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="J12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L12" s="2" t="n">
+        <v>43628</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n">
+        <v>2412</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>506</v>
+      </c>
+      <c r="C13" s="2" t="n">
+        <v>3086</v>
+      </c>
+      <c r="D13" s="3" t="n">
+        <v>328.071052393943</v>
+      </c>
+      <c r="E13" s="3" t="n">
+        <v>90.31164676207929</v>
+      </c>
+      <c r="F13" s="3" t="n">
+        <v>237.7594056318637</v>
+      </c>
+      <c r="G13" s="3" t="n">
+        <v>1.596159631235717</v>
+      </c>
+      <c r="H13" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="I13" s="2" t="n">
+        <v>28</v>
+      </c>
+      <c r="J13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="K13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="L13" s="2" t="n">
+        <v>43594</v>
       </c>
     </row>
   </sheetData>
@@ -4349,7 +7094,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>All three fixed schedules are retained; do not select a seed by outcome.</t>
+          <t>All twelve fixed schedules are retained; do not select a seed by outcome.</t>
         </is>
       </c>
     </row>

</xml_diff>